<commit_message>
Production plan template: owner's corrected version (Desem schema product names match the shop)
</commit_message>
<xml_diff>
--- a/website/templates/production-plan.xlsx
+++ b/website/templates/production-plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sophia/Library/Mobile Documents/com~apple~CloudDocs/Bakery/Production - orders+planning/Deliverable_2026-09/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CA51768-ED83-8644-9379-FEF1C9EA20BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC61A160-7DB9-1A4F-8539-4428E9BACD28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{3B4CC261-C09A-2545-A80C-BE0417D57BA1}"/>
   </bookViews>
@@ -75,7 +75,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="838" uniqueCount="302">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="843" uniqueCount="299">
   <si>
     <t>Datum</t>
   </si>
@@ -258,9 +258,6 @@
   </si>
   <si>
     <t>Wat</t>
-  </si>
-  <si>
-    <t>La Brioche</t>
   </si>
   <si>
     <t>Stockdorf Sourdough</t>
@@ -1078,12 +1075,6 @@
   </si>
   <si>
     <t>Pizzaballen (10x 252gr)</t>
-  </si>
-  <si>
-    <t>Ciabatta - mit oder ohne Oliven</t>
-  </si>
-  <si>
-    <t>Wheat &amp; Rye Sourdough - Roggenmischbrot</t>
   </si>
   <si>
     <t>SL(t)</t>
@@ -1871,7 +1862,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="220">
+  <cellXfs count="219">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2268,6 +2259,13 @@
     </xf>
     <xf numFmtId="166" fontId="53" fillId="7" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="47" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="55" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -2279,14 +2277,6 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="55" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -2715,12 +2705,12 @@
         <v>24</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="B3" s="27" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="C3" s="175">
         <f>SUMIFS(Orders!G:G,Orders!F:F,B3)</f>
@@ -2733,7 +2723,7 @@
     </row>
     <row r="4" spans="1:5">
       <c r="B4" s="27" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C4" s="175">
         <f>SUMIFS(Orders!G:G,Orders!F:F,B4)</f>
@@ -2746,7 +2736,7 @@
     </row>
     <row r="5" spans="1:5">
       <c r="B5" s="27" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="C5" s="175">
         <f>SUMIFS(Orders!G:G,Orders!F:F,B5)</f>
@@ -2759,7 +2749,7 @@
     </row>
     <row r="6" spans="1:5">
       <c r="B6" s="27" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="C6" s="175">
         <f>SUMIFS(Orders!G:G,Orders!F:F,B6)</f>
@@ -2772,7 +2762,7 @@
     </row>
     <row r="7" spans="1:5">
       <c r="B7" s="27" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="C7" s="175">
         <f>SUMIFS(Orders!G:G,Orders!F:F,B7)</f>
@@ -2786,7 +2776,7 @@
     <row r="8" spans="1:5">
       <c r="A8" s="178"/>
       <c r="B8" s="27" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="C8" s="175">
         <f>SUMIFS(Orders!G:G,Orders!F:F,B8)</f>
@@ -2799,7 +2789,7 @@
     </row>
     <row r="9" spans="1:5">
       <c r="B9" s="27" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="C9" s="175">
         <f>SUMIFS(Orders!G:G,Orders!F:F,B9)</f>
@@ -2812,7 +2802,7 @@
     </row>
     <row r="10" spans="1:5">
       <c r="B10" s="27" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="C10" s="175">
         <f>SUMIFS(Orders!G:G,Orders!F:F,B10)</f>
@@ -2825,34 +2815,34 @@
     </row>
     <row r="11" spans="1:5">
       <c r="B11" s="27" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="C11" s="175">
         <f>SUMIFS(Orders!G:G,Orders!F:F,B11)</f>
         <v>0</v>
       </c>
       <c r="D11" s="175">
-        <v>340</v>
+        <v>350</v>
       </c>
       <c r="E11" s="27"/>
     </row>
     <row r="12" spans="1:5">
       <c r="B12" s="181" t="s">
-        <v>276</v>
-      </c>
-      <c r="C12" s="219">
+        <v>275</v>
+      </c>
+      <c r="C12" s="214">
         <v>0</v>
       </c>
       <c r="D12" s="182">
         <v>252</v>
       </c>
       <c r="E12" s="181" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="13" spans="1:5">
       <c r="B13" s="181" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C13" s="182">
         <v>0</v>
@@ -2861,7 +2851,7 @@
         <v>1900</v>
       </c>
       <c r="E13" s="181" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="14" spans="1:5" s="107" customFormat="1">
@@ -2875,12 +2865,12 @@
         <v>80</v>
       </c>
       <c r="E14" s="145" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="15" spans="1:5">
       <c r="B15" s="181" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C15" s="182">
         <v>0</v>
@@ -2889,12 +2879,12 @@
         <v>65</v>
       </c>
       <c r="E15" s="181" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="16" spans="1:5" s="107" customFormat="1">
       <c r="B16" s="145" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C16" s="146">
         <v>0</v>
@@ -2903,12 +2893,12 @@
         <v>120</v>
       </c>
       <c r="E16" s="145" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="17" spans="2:5">
       <c r="B17" s="181" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C17" s="182">
         <v>0</v>
@@ -2917,12 +2907,12 @@
         <v>85</v>
       </c>
       <c r="E17" s="181" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="18" spans="2:5" s="107" customFormat="1">
       <c r="B18" s="145" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C18" s="146">
         <v>0</v>
@@ -2932,12 +2922,12 @@
         <v>504</v>
       </c>
       <c r="E18" s="145" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="19" spans="2:5" s="107" customFormat="1">
       <c r="B19" s="145" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C19" s="146">
         <v>0</v>
@@ -2946,12 +2936,12 @@
         <v>750</v>
       </c>
       <c r="E19" s="145" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="20" spans="2:5" s="107" customFormat="1">
       <c r="B20" s="145" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C20" s="146">
         <v>0</v>
@@ -2960,7 +2950,7 @@
         <v>70</v>
       </c>
       <c r="E20" s="145" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="21" spans="2:5">
@@ -3023,61 +3013,61 @@
         <v>60</v>
       </c>
       <c r="C1" s="151" t="s">
+        <v>198</v>
+      </c>
+      <c r="D1" s="151" t="s">
         <v>199</v>
       </c>
-      <c r="D1" s="151" t="s">
+      <c r="E1" s="151" t="s">
         <v>200</v>
       </c>
-      <c r="E1" s="151" t="s">
-        <v>201</v>
-      </c>
       <c r="F1" s="151" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="2" spans="2:6">
       <c r="B2" s="152" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C2" s="153">
         <f>30+60+60</f>
         <v>150</v>
       </c>
       <c r="D2" s="152" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="E2" s="152" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="F2" s="168"/>
     </row>
     <row r="3" spans="2:6">
       <c r="B3" s="152" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C3" s="153">
         <v>180</v>
       </c>
       <c r="D3" s="152" t="s">
+        <v>249</v>
+      </c>
+      <c r="E3" s="152" t="s">
         <v>250</v>
-      </c>
-      <c r="E3" s="152" t="s">
-        <v>251</v>
       </c>
       <c r="F3" s="168"/>
     </row>
     <row r="4" spans="2:6">
       <c r="B4" s="152" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C4" s="153">
         <v>1355</v>
       </c>
       <c r="D4" s="152" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="E4" s="152" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F4" s="168">
         <v>790</v>
@@ -3085,32 +3075,32 @@
     </row>
     <row r="5" spans="2:6">
       <c r="B5" s="152" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C5" s="153">
         <f>40+80+160</f>
         <v>280</v>
       </c>
       <c r="D5" s="152" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="E5" s="152" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F5" s="168"/>
     </row>
     <row r="6" spans="2:6">
       <c r="B6" s="152" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C6" s="153">
         <v>1200</v>
       </c>
       <c r="D6" s="152" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="E6" s="152" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="F6" s="168"/>
     </row>
@@ -3118,7 +3108,7 @@
       <c r="B7" s="152"/>
       <c r="C7" s="153"/>
       <c r="D7" s="152" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="E7" s="152"/>
       <c r="F7" s="168">
@@ -3129,7 +3119,7 @@
       <c r="B8" s="152"/>
       <c r="C8" s="153"/>
       <c r="D8" s="152" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="E8" s="152"/>
       <c r="F8" s="168">
@@ -3138,13 +3128,13 @@
     </row>
     <row r="9" spans="2:6">
       <c r="B9" s="152" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C9" s="153">
         <v>1802</v>
       </c>
       <c r="D9" s="152" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="E9" s="152"/>
       <c r="F9" s="168"/>
@@ -3443,7 +3433,7 @@
         <v>#N/A</v>
       </c>
       <c r="P2" s="86" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="Q2" s="89">
         <f t="shared" ref="Q2" si="0">Q3/C2*1000</f>
@@ -3487,28 +3477,28 @@
         <v>30</v>
       </c>
       <c r="C3" s="90" t="s">
+        <v>138</v>
+      </c>
+      <c r="D3" s="90" t="s">
+        <v>90</v>
+      </c>
+      <c r="E3" s="90" t="s">
+        <v>106</v>
+      </c>
+      <c r="F3" s="90" t="s">
         <v>139</v>
       </c>
-      <c r="D3" s="90" t="s">
-        <v>91</v>
-      </c>
-      <c r="E3" s="90" t="s">
-        <v>107</v>
-      </c>
-      <c r="F3" s="90" t="s">
+      <c r="G3" s="90" t="s">
         <v>140</v>
       </c>
-      <c r="G3" s="90" t="s">
+      <c r="H3" s="90" t="s">
         <v>141</v>
       </c>
-      <c r="H3" s="90" t="s">
-        <v>142</v>
-      </c>
       <c r="I3" s="90" t="s">
+        <v>143</v>
+      </c>
+      <c r="J3" s="90" t="s">
         <v>144</v>
-      </c>
-      <c r="J3" s="90" t="s">
-        <v>145</v>
       </c>
       <c r="K3" s="90"/>
       <c r="O3" s="91"/>
@@ -3642,7 +3632,7 @@
     </row>
     <row r="5" spans="2:38">
       <c r="B5" s="99" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C5" s="100"/>
       <c r="D5" s="100">
@@ -3717,7 +3707,7 @@
     </row>
     <row r="6" spans="2:38">
       <c r="B6" s="99" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C6" s="100">
         <v>3</v>
@@ -3851,7 +3841,7 @@
     </row>
     <row r="8" spans="2:38">
       <c r="B8" s="99" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C8" s="100"/>
       <c r="D8" s="100"/>
@@ -4194,7 +4184,7 @@
     </row>
     <row r="13" spans="2:38">
       <c r="B13" s="99" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C13" s="100">
         <v>5</v>
@@ -4393,7 +4383,7 @@
     </row>
     <row r="16" spans="2:38">
       <c r="B16" s="99" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C16" s="100"/>
       <c r="D16" s="100"/>
@@ -4458,7 +4448,7 @@
     </row>
     <row r="17" spans="2:27">
       <c r="B17" s="99" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C17" s="100"/>
       <c r="D17" s="100"/>
@@ -4663,7 +4653,7 @@
     </row>
     <row r="20" spans="2:27">
       <c r="B20" s="99" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C20" s="100"/>
       <c r="D20" s="100">
@@ -4731,7 +4721,7 @@
     </row>
     <row r="21" spans="2:27">
       <c r="B21" s="99" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C21" s="100"/>
       <c r="D21" s="100">
@@ -4796,7 +4786,7 @@
     </row>
     <row r="22" spans="2:27">
       <c r="B22" s="99" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C22" s="100"/>
       <c r="D22" s="100"/>
@@ -4861,7 +4851,7 @@
     </row>
     <row r="23" spans="2:27">
       <c r="B23" s="99" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C23" s="100"/>
       <c r="D23" s="100"/>
@@ -4926,7 +4916,7 @@
     </row>
     <row r="24" spans="2:27">
       <c r="B24" s="99" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C24" s="100"/>
       <c r="D24" s="100"/>
@@ -4991,7 +4981,7 @@
     </row>
     <row r="25" spans="2:27">
       <c r="B25" s="99" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C25" s="100"/>
       <c r="D25" s="100"/>
@@ -5058,7 +5048,7 @@
     </row>
     <row r="26" spans="2:27">
       <c r="B26" s="106" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C26" s="100">
         <v>2</v>
@@ -5125,7 +5115,7 @@
     </row>
     <row r="27" spans="2:27">
       <c r="B27" s="106" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C27" s="100"/>
       <c r="D27" s="100"/>
@@ -5190,7 +5180,7 @@
     </row>
     <row r="28" spans="2:27">
       <c r="B28" s="106" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C28" s="100"/>
       <c r="D28" s="100"/>
@@ -5255,7 +5245,7 @@
     </row>
     <row r="29" spans="2:27">
       <c r="B29" s="99" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C29" s="100"/>
       <c r="D29" s="100"/>
@@ -5320,7 +5310,7 @@
     </row>
     <row r="30" spans="2:27">
       <c r="B30" s="99" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C30" s="100">
         <v>8</v>
@@ -5454,7 +5444,7 @@
     </row>
     <row r="32" spans="2:27">
       <c r="B32" s="99" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C32" s="100"/>
       <c r="D32" s="100"/>
@@ -5519,7 +5509,7 @@
     </row>
     <row r="33" spans="2:27">
       <c r="B33" s="99" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C33" s="100"/>
       <c r="D33" s="100"/>
@@ -5584,7 +5574,7 @@
     </row>
     <row r="34" spans="2:27">
       <c r="B34" s="99" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C34" s="100">
         <v>147</v>
@@ -5655,7 +5645,7 @@
     </row>
     <row r="35" spans="2:27">
       <c r="B35" s="99" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C35" s="100"/>
       <c r="D35" s="100"/>
@@ -5724,7 +5714,7 @@
     </row>
     <row r="36" spans="2:27">
       <c r="B36" s="99" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C36" s="100"/>
       <c r="D36" s="100">
@@ -5797,7 +5787,7 @@
     </row>
     <row r="37" spans="2:27">
       <c r="B37" s="99" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C37" s="100"/>
       <c r="D37" s="100"/>
@@ -5927,7 +5917,7 @@
     </row>
     <row r="39" spans="2:27">
       <c r="B39" s="99" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C39" s="100">
         <v>1</v>
@@ -6203,7 +6193,7 @@
     </row>
     <row r="43" spans="2:27">
       <c r="B43" s="99" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C43" s="100"/>
       <c r="D43" s="100"/>
@@ -6270,7 +6260,7 @@
     </row>
     <row r="44" spans="2:27">
       <c r="B44" s="99" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C44" s="100">
         <v>1</v>
@@ -6414,7 +6404,7 @@
     </row>
     <row r="46" spans="2:27">
       <c r="B46" s="99" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C46" s="100"/>
       <c r="D46" s="100"/>
@@ -6603,7 +6593,7 @@
       </c>
     </row>
     <row r="10" spans="2:5">
-      <c r="B10" s="213" t="s">
+      <c r="B10" s="216" t="s">
         <v>48</v>
       </c>
       <c r="C10" s="27" t="s">
@@ -6617,7 +6607,7 @@
       </c>
     </row>
     <row r="11" spans="2:5" ht="34">
-      <c r="B11" s="214"/>
+      <c r="B11" s="217"/>
       <c r="C11" s="34" t="s">
         <v>47</v>
       </c>
@@ -6629,7 +6619,7 @@
       </c>
     </row>
     <row r="12" spans="2:5">
-      <c r="B12" s="215"/>
+      <c r="B12" s="218"/>
       <c r="C12" s="27" t="s">
         <v>25</v>
       </c>
@@ -6650,7 +6640,7 @@
       <c r="E14" s="31"/>
     </row>
     <row r="15" spans="2:5">
-      <c r="B15" s="212" t="s">
+      <c r="B15" s="215" t="s">
         <v>43</v>
       </c>
       <c r="C15" s="27" t="s">
@@ -6662,7 +6652,7 @@
       <c r="E15" s="29"/>
     </row>
     <row r="16" spans="2:5">
-      <c r="B16" s="212"/>
+      <c r="B16" s="215"/>
       <c r="C16" s="27" t="s">
         <v>42</v>
       </c>
@@ -6800,7 +6790,7 @@
         <v>#N/A</v>
       </c>
       <c r="P2" s="86" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="Q2" s="89">
         <f t="shared" ref="Q2:Y2" si="0">Q3/C2*1000</f>
@@ -6844,10 +6834,10 @@
         <v>30</v>
       </c>
       <c r="C3" s="90" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D3" s="90" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E3" s="90" t="s">
         <v>25</v>
@@ -6989,7 +6979,7 @@
     </row>
     <row r="5" spans="2:38">
       <c r="B5" s="99" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C5" s="100"/>
       <c r="D5" s="100"/>
@@ -7056,7 +7046,7 @@
     </row>
     <row r="6" spans="2:38">
       <c r="B6" s="99" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C6" s="100"/>
       <c r="D6" s="100"/>
@@ -7188,7 +7178,7 @@
     </row>
     <row r="8" spans="2:38">
       <c r="B8" s="99" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C8" s="100"/>
       <c r="D8" s="100"/>
@@ -7517,7 +7507,7 @@
     </row>
     <row r="13" spans="2:38">
       <c r="B13" s="99" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C13" s="100"/>
       <c r="D13" s="100"/>
@@ -7714,7 +7704,7 @@
     </row>
     <row r="16" spans="2:38">
       <c r="B16" s="99" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C16" s="100"/>
       <c r="D16" s="100"/>
@@ -7779,7 +7769,7 @@
     </row>
     <row r="17" spans="2:27">
       <c r="B17" s="99" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C17" s="100"/>
       <c r="D17" s="100"/>
@@ -7974,7 +7964,7 @@
     </row>
     <row r="20" spans="2:27">
       <c r="B20" s="99" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C20" s="100"/>
       <c r="D20" s="100"/>
@@ -8040,7 +8030,7 @@
     </row>
     <row r="21" spans="2:27">
       <c r="B21" s="99" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C21" s="100"/>
       <c r="D21" s="100"/>
@@ -8103,7 +8093,7 @@
     </row>
     <row r="22" spans="2:27">
       <c r="B22" s="99" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C22" s="100"/>
       <c r="D22" s="100"/>
@@ -8168,7 +8158,7 @@
     </row>
     <row r="23" spans="2:27">
       <c r="B23" s="99" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C23" s="100"/>
       <c r="D23" s="100"/>
@@ -8233,7 +8223,7 @@
     </row>
     <row r="24" spans="2:27">
       <c r="B24" s="99" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C24" s="100"/>
       <c r="D24" s="100"/>
@@ -8298,7 +8288,7 @@
     </row>
     <row r="25" spans="2:27">
       <c r="B25" s="99" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C25" s="100"/>
       <c r="D25" s="100"/>
@@ -8361,7 +8351,7 @@
     </row>
     <row r="26" spans="2:27">
       <c r="B26" s="106" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C26" s="100"/>
       <c r="D26" s="100"/>
@@ -8426,7 +8416,7 @@
     </row>
     <row r="27" spans="2:27">
       <c r="B27" s="106" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C27" s="100"/>
       <c r="D27" s="100"/>
@@ -8491,7 +8481,7 @@
     </row>
     <row r="28" spans="2:27">
       <c r="B28" s="106" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C28" s="100"/>
       <c r="D28" s="100"/>
@@ -8556,7 +8546,7 @@
     </row>
     <row r="29" spans="2:27">
       <c r="B29" s="99" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C29" s="100"/>
       <c r="D29" s="100"/>
@@ -8621,7 +8611,7 @@
     </row>
     <row r="30" spans="2:27">
       <c r="B30" s="99" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C30" s="100"/>
       <c r="D30" s="100"/>
@@ -8751,7 +8741,7 @@
     </row>
     <row r="32" spans="2:27">
       <c r="B32" s="99" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C32" s="100"/>
       <c r="D32" s="100"/>
@@ -8816,7 +8806,7 @@
     </row>
     <row r="33" spans="2:27">
       <c r="B33" s="99" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C33" s="100"/>
       <c r="D33" s="100"/>
@@ -8881,7 +8871,7 @@
     </row>
     <row r="34" spans="2:27">
       <c r="B34" s="99" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C34" s="100"/>
       <c r="D34" s="100"/>
@@ -8946,7 +8936,7 @@
     </row>
     <row r="35" spans="2:27">
       <c r="B35" s="99" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C35" s="100"/>
       <c r="D35" s="100"/>
@@ -9011,7 +9001,7 @@
     </row>
     <row r="36" spans="2:27">
       <c r="B36" s="99" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C36" s="100"/>
       <c r="D36" s="100"/>
@@ -9076,7 +9066,7 @@
     </row>
     <row r="37" spans="2:27">
       <c r="B37" s="99" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C37" s="100"/>
       <c r="D37" s="100"/>
@@ -9206,7 +9196,7 @@
     </row>
     <row r="39" spans="2:27">
       <c r="B39" s="99" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C39" s="100"/>
       <c r="D39" s="100"/>
@@ -9466,7 +9456,7 @@
     </row>
     <row r="43" spans="2:27">
       <c r="B43" s="99" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C43" s="100"/>
       <c r="D43" s="100"/>
@@ -9531,7 +9521,7 @@
     </row>
     <row r="44" spans="2:27">
       <c r="B44" s="99" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C44" s="100"/>
       <c r="D44" s="100"/>
@@ -9659,7 +9649,7 @@
     </row>
     <row r="46" spans="2:27">
       <c r="B46" s="99" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C46" s="100"/>
       <c r="D46" s="100"/>
@@ -9806,56 +9796,56 @@
   <sheetPr>
     <tabColor theme="2" tint="-9.9978637043366805E-2"/>
   </sheetPr>
-  <dimension ref="A1:X38"/>
+  <dimension ref="A1:Q38"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col min="1" max="1" width="13.5" style="216" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12" style="216" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.1640625" style="216" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8" style="216" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.83203125" style="216" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="21.1640625" style="216" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.5" style="216" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.83203125" style="216" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="26" style="216" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.6640625" style="216" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.5" style="216" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.6640625" style="216" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="6.33203125" style="216" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="7.5" style="216" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="20.1640625" style="216" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="9.83203125" style="216" customWidth="1"/>
-    <col min="17" max="17" width="15.5" style="217" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="36.1640625" style="216" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="14.1640625" style="216" customWidth="1"/>
-    <col min="20" max="20" width="12.6640625" style="216" customWidth="1"/>
-    <col min="21" max="21" width="36.1640625" style="216" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="22.5" style="216" customWidth="1"/>
-    <col min="23" max="23" width="14.5" style="216" customWidth="1"/>
-    <col min="24" max="24" width="22.33203125" style="216" customWidth="1"/>
-    <col min="25" max="25" width="22.1640625" style="216" customWidth="1"/>
-    <col min="26" max="27" width="13.83203125" style="216" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="9.83203125" style="216" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="9" style="216" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="13.5" style="216" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="13" style="216" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="11.5" style="216" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="13.1640625" style="216" bestFit="1" customWidth="1"/>
-    <col min="34" max="35" width="15.6640625" style="216" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="11.6640625" style="216" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="10.83203125" style="216"/>
-    <col min="38" max="38" width="15.33203125" style="216" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="14.83203125" style="216" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="13.33203125" style="216" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="11.5" style="216" bestFit="1" customWidth="1"/>
-    <col min="42" max="43" width="12" style="216" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="13.1640625" style="216" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="20" style="216" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="6.5" style="216" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="82.33203125" style="216" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="14.6640625" style="216" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="36" style="216" bestFit="1" customWidth="1"/>
-    <col min="50" max="16384" width="10.83203125" style="216"/>
+    <col min="1" max="1" width="13.5" style="57" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12" style="57" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.1640625" style="57" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8" style="57" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.83203125" style="57" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21.1640625" style="57" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.5" style="57" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.83203125" style="57" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="26" style="57" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.6640625" style="57" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.5" style="57" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.6640625" style="57" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="6.33203125" style="57" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="7.5" style="57" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="20.1640625" style="57" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="9.83203125" style="57" customWidth="1"/>
+    <col min="17" max="17" width="15.5" style="212" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="36.1640625" style="57" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="14.1640625" style="57" customWidth="1"/>
+    <col min="20" max="20" width="12.6640625" style="57" customWidth="1"/>
+    <col min="21" max="21" width="36.1640625" style="57" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="22.5" style="57" customWidth="1"/>
+    <col min="23" max="23" width="14.5" style="57" customWidth="1"/>
+    <col min="24" max="24" width="22.33203125" style="57" customWidth="1"/>
+    <col min="25" max="25" width="22.1640625" style="57" customWidth="1"/>
+    <col min="26" max="27" width="13.83203125" style="57" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="9.83203125" style="57" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="9" style="57" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="13.5" style="57" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="13" style="57" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="11.5" style="57" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="13.1640625" style="57" bestFit="1" customWidth="1"/>
+    <col min="34" max="35" width="15.6640625" style="57" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="11.6640625" style="57" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="10.83203125" style="57"/>
+    <col min="38" max="38" width="15.33203125" style="57" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="14.83203125" style="57" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="13.33203125" style="57" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="11.5" style="57" bestFit="1" customWidth="1"/>
+    <col min="42" max="43" width="12" style="57" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="13.1640625" style="57" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="20" style="57" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="6.5" style="57" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="82.33203125" style="57" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="14.6640625" style="57" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="36" style="57" bestFit="1" customWidth="1"/>
+    <col min="50" max="16384" width="10.83203125" style="57"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15">
@@ -9877,8 +9867,8 @@
     </row>
     <row r="2" spans="1:15">
       <c r="A2"/>
-      <c r="B2" s="218"/>
-      <c r="C2" s="218"/>
+      <c r="B2" s="213"/>
+      <c r="C2" s="213"/>
       <c r="D2"/>
       <c r="E2"/>
       <c r="F2"/>
@@ -9894,8 +9884,8 @@
     </row>
     <row r="3" spans="1:15">
       <c r="A3"/>
-      <c r="B3" s="218"/>
-      <c r="C3" s="218"/>
+      <c r="B3" s="213"/>
+      <c r="C3" s="213"/>
       <c r="D3"/>
       <c r="E3"/>
       <c r="F3"/>
@@ -9911,8 +9901,8 @@
     </row>
     <row r="4" spans="1:15">
       <c r="A4"/>
-      <c r="B4" s="218"/>
-      <c r="C4" s="218"/>
+      <c r="B4" s="213"/>
+      <c r="C4" s="213"/>
       <c r="D4"/>
       <c r="E4"/>
       <c r="F4"/>
@@ -9928,8 +9918,8 @@
     </row>
     <row r="5" spans="1:15">
       <c r="A5"/>
-      <c r="B5" s="218"/>
-      <c r="C5" s="218"/>
+      <c r="B5" s="213"/>
+      <c r="C5" s="213"/>
       <c r="D5"/>
       <c r="E5"/>
       <c r="F5"/>
@@ -9945,8 +9935,8 @@
     </row>
     <row r="6" spans="1:15">
       <c r="A6"/>
-      <c r="B6" s="218"/>
-      <c r="C6" s="218"/>
+      <c r="B6" s="213"/>
+      <c r="C6" s="213"/>
       <c r="D6"/>
       <c r="E6"/>
       <c r="F6"/>
@@ -9962,8 +9952,8 @@
     </row>
     <row r="7" spans="1:15">
       <c r="A7"/>
-      <c r="B7" s="218"/>
-      <c r="C7" s="218"/>
+      <c r="B7" s="213"/>
+      <c r="C7" s="213"/>
       <c r="D7"/>
       <c r="E7"/>
       <c r="F7"/>
@@ -9979,8 +9969,8 @@
     </row>
     <row r="8" spans="1:15">
       <c r="A8"/>
-      <c r="B8" s="218"/>
-      <c r="C8" s="218"/>
+      <c r="B8" s="213"/>
+      <c r="C8" s="213"/>
       <c r="D8"/>
       <c r="E8"/>
       <c r="F8"/>
@@ -9996,8 +9986,8 @@
     </row>
     <row r="9" spans="1:15">
       <c r="A9"/>
-      <c r="B9" s="218"/>
-      <c r="C9" s="218"/>
+      <c r="B9" s="213"/>
+      <c r="C9" s="213"/>
       <c r="D9"/>
       <c r="E9"/>
       <c r="F9"/>
@@ -10013,8 +10003,8 @@
     </row>
     <row r="10" spans="1:15">
       <c r="A10"/>
-      <c r="B10" s="218"/>
-      <c r="C10" s="218"/>
+      <c r="B10" s="213"/>
+      <c r="C10" s="213"/>
       <c r="D10"/>
       <c r="E10"/>
       <c r="F10"/>
@@ -10030,8 +10020,8 @@
     </row>
     <row r="11" spans="1:15">
       <c r="A11"/>
-      <c r="B11" s="218"/>
-      <c r="C11" s="218"/>
+      <c r="B11" s="213"/>
+      <c r="C11" s="213"/>
       <c r="D11"/>
       <c r="E11"/>
       <c r="F11"/>
@@ -10047,8 +10037,8 @@
     </row>
     <row r="12" spans="1:15">
       <c r="A12"/>
-      <c r="B12" s="218"/>
-      <c r="C12" s="218"/>
+      <c r="B12" s="213"/>
+      <c r="C12" s="213"/>
       <c r="D12"/>
       <c r="E12"/>
       <c r="F12"/>
@@ -10064,8 +10054,8 @@
     </row>
     <row r="13" spans="1:15">
       <c r="A13"/>
-      <c r="B13" s="218"/>
-      <c r="C13" s="218"/>
+      <c r="B13" s="213"/>
+      <c r="C13" s="213"/>
       <c r="D13"/>
       <c r="E13"/>
       <c r="F13"/>
@@ -10081,8 +10071,8 @@
     </row>
     <row r="14" spans="1:15">
       <c r="A14"/>
-      <c r="B14" s="218"/>
-      <c r="C14" s="218"/>
+      <c r="B14" s="213"/>
+      <c r="C14" s="213"/>
       <c r="D14"/>
       <c r="E14"/>
       <c r="F14"/>
@@ -10098,8 +10088,8 @@
     </row>
     <row r="15" spans="1:15">
       <c r="A15"/>
-      <c r="B15" s="218"/>
-      <c r="C15" s="218"/>
+      <c r="B15" s="213"/>
+      <c r="C15" s="213"/>
       <c r="D15"/>
       <c r="E15"/>
       <c r="F15"/>
@@ -10115,8 +10105,8 @@
     </row>
     <row r="16" spans="1:15">
       <c r="A16"/>
-      <c r="B16" s="218"/>
-      <c r="C16" s="218"/>
+      <c r="B16" s="213"/>
+      <c r="C16" s="213"/>
       <c r="D16"/>
       <c r="E16"/>
       <c r="F16"/>
@@ -10132,8 +10122,8 @@
     </row>
     <row r="17" spans="1:15">
       <c r="A17"/>
-      <c r="B17" s="218"/>
-      <c r="C17" s="218"/>
+      <c r="B17" s="213"/>
+      <c r="C17" s="213"/>
       <c r="D17"/>
       <c r="E17"/>
       <c r="F17"/>
@@ -10205,7 +10195,7 @@
   <sheetPr>
     <tabColor theme="2" tint="-9.9978637043366805E-2"/>
   </sheetPr>
-  <dimension ref="B1:O38"/>
+  <dimension ref="B1:O40"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="3.33203125" style="201" customWidth="1"/>
@@ -10233,13 +10223,13 @@
       <c r="B2" s="194"/>
       <c r="C2" s="194"/>
       <c r="D2" s="194" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="E2" s="194" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="F2" s="194" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="G2" s="183"/>
       <c r="H2" s="183"/>
@@ -10253,10 +10243,10 @@
     </row>
     <row r="3" spans="2:15">
       <c r="B3" s="197" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C3" s="198" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="D3" s="198">
         <f>F3*E3</f>
@@ -10281,10 +10271,10 @@
     </row>
     <row r="4" spans="2:15" s="166" customFormat="1">
       <c r="B4" s="197" t="s">
-        <v>278</v>
+        <v>297</v>
       </c>
       <c r="C4" s="198" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="D4" s="198">
         <f>F4*E4</f>
@@ -10309,10 +10299,10 @@
     </row>
     <row r="5" spans="2:15">
       <c r="B5" s="197" t="s">
-        <v>277</v>
+        <v>294</v>
       </c>
       <c r="C5" s="198" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="D5" s="198">
         <f>F5*E5</f>
@@ -10322,7 +10312,7 @@
         <v>65</v>
       </c>
       <c r="F5" s="198">
-        <f>SUMIF(Overview!B3:B11,'Desem schema'!B5,Overview!C3:C11)</f>
+        <f>SUMIF(Overview!B1:B9,'Desem schema'!B5,Overview!C1:C9)</f>
         <v>0</v>
       </c>
       <c r="G5" s="202"/>
@@ -10337,20 +10327,20 @@
     </row>
     <row r="6" spans="2:15">
       <c r="B6" s="197" t="s">
-        <v>61</v>
+        <v>295</v>
       </c>
       <c r="C6" s="198" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="D6" s="198">
         <f>F6*E6</f>
         <v>0</v>
       </c>
       <c r="E6" s="198">
-        <v>15</v>
+        <v>65</v>
       </c>
       <c r="F6" s="198">
-        <f>SUMIF(Overview!B3:B11,'Desem schema'!B6,Overview!C3:C11)</f>
+        <f>SUMIF(Overview!B2:B10,'Desem schema'!B6,Overview!C2:C10)</f>
         <v>0</v>
       </c>
       <c r="G6" s="202"/>
@@ -10365,12 +10355,22 @@
     </row>
     <row r="7" spans="2:15">
       <c r="B7" s="197" t="s">
-        <v>255</v>
-      </c>
-      <c r="C7" s="198"/>
-      <c r="D7" s="198"/>
-      <c r="E7" s="198"/>
-      <c r="F7" s="198"/>
+        <v>296</v>
+      </c>
+      <c r="C7" s="198" t="s">
+        <v>276</v>
+      </c>
+      <c r="D7" s="198">
+        <f>F7*E7</f>
+        <v>0</v>
+      </c>
+      <c r="E7" s="198">
+        <v>65</v>
+      </c>
+      <c r="F7" s="198">
+        <f>SUMIF(Overview!B3:B11,'Desem schema'!B7,Overview!C3:C11)</f>
+        <v>0</v>
+      </c>
       <c r="G7" s="202"/>
       <c r="H7" s="202"/>
       <c r="I7" s="202"/>
@@ -10382,11 +10382,23 @@
       <c r="O7" s="202"/>
     </row>
     <row r="8" spans="2:15">
-      <c r="B8" s="23"/>
-      <c r="C8" s="156"/>
-      <c r="D8" s="156"/>
-      <c r="E8" s="202"/>
-      <c r="F8" s="202"/>
+      <c r="B8" s="197" t="s">
+        <v>291</v>
+      </c>
+      <c r="C8" s="198" t="s">
+        <v>276</v>
+      </c>
+      <c r="D8" s="198">
+        <f>F8*E8</f>
+        <v>0</v>
+      </c>
+      <c r="E8" s="198">
+        <v>15</v>
+      </c>
+      <c r="F8" s="198">
+        <f>SUMIF(Overview!B3:B11,'Desem schema'!B8,Overview!C3:C11)</f>
+        <v>0</v>
+      </c>
       <c r="G8" s="202"/>
       <c r="H8" s="202"/>
       <c r="I8" s="202"/>
@@ -10397,80 +10409,94 @@
       <c r="N8" s="202"/>
       <c r="O8" s="202"/>
     </row>
-    <row r="9" spans="2:15" s="166" customFormat="1">
-      <c r="C9" s="194" t="s">
-        <v>126</v>
-      </c>
-      <c r="D9" s="195"/>
-      <c r="E9" s="184"/>
-      <c r="G9" s="184"/>
-      <c r="H9" s="184"/>
-      <c r="I9" s="184"/>
-      <c r="J9" s="184"/>
-      <c r="K9" s="184"/>
-      <c r="L9" s="184"/>
-      <c r="M9" s="184"/>
-      <c r="N9" s="184"/>
-      <c r="O9" s="184"/>
+    <row r="9" spans="2:15">
+      <c r="B9" s="197" t="s">
+        <v>254</v>
+      </c>
+      <c r="C9" s="198" t="s">
+        <v>276</v>
+      </c>
+      <c r="D9" s="198">
+        <f>F9*E9</f>
+        <v>0</v>
+      </c>
+      <c r="E9" s="198">
+        <v>25</v>
+      </c>
+      <c r="F9" s="198">
+        <f>SUMIF(Overview!B4:B12,'Desem schema'!B9,Overview!C4:C12)</f>
+        <v>0</v>
+      </c>
+      <c r="G9" s="202"/>
+      <c r="H9" s="202"/>
+      <c r="I9" s="202"/>
+      <c r="J9" s="202"/>
+      <c r="K9" s="202"/>
+      <c r="L9" s="202"/>
+      <c r="M9" s="202"/>
+      <c r="N9" s="202"/>
+      <c r="O9" s="202"/>
     </row>
     <row r="10" spans="2:15">
-      <c r="C10" s="196" t="s">
-        <v>279</v>
-      </c>
-      <c r="D10" s="196">
-        <f>SUMIF($C$3:$C$7,C10,$D$3:$D$7)</f>
-        <v>0</v>
-      </c>
-      <c r="E10" s="183"/>
-      <c r="G10" s="183"/>
-      <c r="H10" s="183"/>
-      <c r="I10" s="183"/>
-      <c r="J10" s="183"/>
-      <c r="K10" s="183"/>
-      <c r="L10" s="183"/>
-      <c r="M10" s="183"/>
-      <c r="N10" s="183"/>
-      <c r="O10" s="183"/>
-    </row>
-    <row r="11" spans="2:15">
-      <c r="C11" s="196" t="s">
-        <v>280</v>
-      </c>
-      <c r="D11" s="196">
-        <f>SUMIF($C$3:$C$7,C11,$D$3:$D$7)</f>
-        <v>0</v>
-      </c>
-      <c r="E11" s="202"/>
-      <c r="G11" s="202"/>
-      <c r="H11" s="202"/>
-      <c r="I11" s="202"/>
-      <c r="J11" s="202"/>
-      <c r="K11" s="202"/>
-      <c r="L11" s="202"/>
-      <c r="M11" s="202"/>
-      <c r="N11" s="202"/>
-      <c r="O11" s="202"/>
+      <c r="B10" s="23"/>
+      <c r="C10" s="156"/>
+      <c r="D10" s="156"/>
+      <c r="E10" s="202"/>
+      <c r="F10" s="202"/>
+      <c r="G10" s="202"/>
+      <c r="H10" s="202"/>
+      <c r="I10" s="202"/>
+      <c r="J10" s="202"/>
+      <c r="K10" s="202"/>
+      <c r="L10" s="202"/>
+      <c r="M10" s="202"/>
+      <c r="N10" s="202"/>
+      <c r="O10" s="202"/>
+    </row>
+    <row r="11" spans="2:15" s="166" customFormat="1">
+      <c r="C11" s="194" t="s">
+        <v>125</v>
+      </c>
+      <c r="D11" s="195"/>
+      <c r="E11" s="184"/>
+      <c r="G11" s="184"/>
+      <c r="H11" s="184"/>
+      <c r="I11" s="184"/>
+      <c r="J11" s="184"/>
+      <c r="K11" s="184"/>
+      <c r="L11" s="184"/>
+      <c r="M11" s="184"/>
+      <c r="N11" s="184"/>
+      <c r="O11" s="184"/>
     </row>
     <row r="12" spans="2:15">
-      <c r="C12" s="28"/>
-      <c r="D12" s="28"/>
-      <c r="E12" s="202"/>
-      <c r="G12" s="202"/>
-      <c r="H12" s="202"/>
-      <c r="I12" s="202"/>
-      <c r="J12" s="202"/>
-      <c r="K12" s="202"/>
-      <c r="L12" s="202"/>
-      <c r="M12" s="202"/>
-      <c r="N12" s="202"/>
-      <c r="O12" s="202"/>
+      <c r="C12" s="196" t="s">
+        <v>276</v>
+      </c>
+      <c r="D12" s="196">
+        <f>SUMIF($C$3:$C$9,C12,$D$3:$D$9)</f>
+        <v>0</v>
+      </c>
+      <c r="E12" s="183"/>
+      <c r="G12" s="183"/>
+      <c r="H12" s="183"/>
+      <c r="I12" s="183"/>
+      <c r="J12" s="183"/>
+      <c r="K12" s="183"/>
+      <c r="L12" s="183"/>
+      <c r="M12" s="183"/>
+      <c r="N12" s="183"/>
+      <c r="O12" s="183"/>
     </row>
     <row r="13" spans="2:15">
-      <c r="B13" s="23"/>
-      <c r="C13" s="156"/>
-      <c r="D13" s="156"/>
+      <c r="C13" s="196" t="s">
+        <v>277</v>
+      </c>
+      <c r="D13" s="196">
+        <f>SUMIF($C$3:$C$9,C13,$D$3:$D$9)</f>
+        <v>0</v>
+      </c>
       <c r="E13" s="202"/>
-      <c r="F13" s="202"/>
       <c r="G13" s="202"/>
       <c r="H13" s="202"/>
       <c r="I13" s="202"/>
@@ -10482,11 +10508,9 @@
       <c r="O13" s="202"/>
     </row>
     <row r="14" spans="2:15">
-      <c r="B14" s="23"/>
-      <c r="C14" s="156"/>
-      <c r="D14" s="156"/>
+      <c r="C14" s="28"/>
+      <c r="D14" s="28"/>
       <c r="E14" s="202"/>
-      <c r="F14" s="202"/>
       <c r="G14" s="202"/>
       <c r="H14" s="202"/>
       <c r="I14" s="202"/>
@@ -10498,384 +10522,416 @@
       <c r="O14" s="202"/>
     </row>
     <row r="15" spans="2:15">
-      <c r="D15" s="203" t="s">
-        <v>291</v>
-      </c>
-      <c r="E15" s="204" t="s">
-        <v>289</v>
-      </c>
-      <c r="F15" s="204" t="s">
+      <c r="B15" s="23"/>
+      <c r="C15" s="156"/>
+      <c r="D15" s="156"/>
+      <c r="E15" s="202"/>
+      <c r="F15" s="202"/>
+      <c r="G15" s="202"/>
+      <c r="H15" s="202"/>
+      <c r="I15" s="202"/>
+      <c r="J15" s="202"/>
+      <c r="K15" s="202"/>
+      <c r="L15" s="202"/>
+      <c r="M15" s="202"/>
+      <c r="N15" s="202"/>
+      <c r="O15" s="202"/>
+    </row>
+    <row r="16" spans="2:15">
+      <c r="B16" s="23"/>
+      <c r="C16" s="156"/>
+      <c r="D16" s="156"/>
+      <c r="E16" s="202"/>
+      <c r="F16" s="202"/>
+      <c r="G16" s="202"/>
+      <c r="H16" s="202"/>
+      <c r="I16" s="202"/>
+      <c r="J16" s="202"/>
+      <c r="K16" s="202"/>
+      <c r="L16" s="202"/>
+      <c r="M16" s="202"/>
+      <c r="N16" s="202"/>
+      <c r="O16" s="202"/>
+    </row>
+    <row r="17" spans="2:15">
+      <c r="D17" s="203" t="s">
+        <v>288</v>
+      </c>
+      <c r="E17" s="204" t="s">
+        <v>286</v>
+      </c>
+      <c r="F17" s="204" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="18" spans="2:15">
+      <c r="B18" s="190" t="s">
+        <v>281</v>
+      </c>
+      <c r="C18" s="199" t="s">
+        <v>276</v>
+      </c>
+      <c r="D18" s="205"/>
+      <c r="E18" s="205"/>
+      <c r="F18" s="191">
+        <f>G18</f>
+        <v>0</v>
+      </c>
+      <c r="G18" s="191">
+        <f>$D$12</f>
+        <v>0</v>
+      </c>
+      <c r="H18" s="23" t="s">
+        <v>280</v>
+      </c>
+      <c r="I18" s="23"/>
+      <c r="J18" s="23" t="s">
         <v>290</v>
       </c>
-    </row>
-    <row r="16" spans="2:15">
-      <c r="B16" s="190" t="s">
-        <v>284</v>
-      </c>
-      <c r="C16" s="199" t="s">
-        <v>279</v>
-      </c>
-      <c r="D16" s="205"/>
-      <c r="E16" s="205"/>
-      <c r="F16" s="191">
-        <f>G16</f>
-        <v>0</v>
-      </c>
-      <c r="G16" s="191">
-        <f>$D$10</f>
-        <v>0</v>
-      </c>
-      <c r="H16" s="23" t="s">
-        <v>283</v>
-      </c>
-      <c r="I16" s="23"/>
-      <c r="J16" s="23" t="s">
-        <v>293</v>
-      </c>
-      <c r="K16" s="23">
-        <f>F16</f>
-        <v>0</v>
-      </c>
-      <c r="M16" s="23"/>
-      <c r="N16" s="23"/>
-      <c r="O16" s="23"/>
-    </row>
-    <row r="17" spans="2:15">
-      <c r="B17" s="197"/>
-      <c r="C17" s="198"/>
-      <c r="D17" s="197"/>
-      <c r="E17" s="197"/>
-      <c r="F17" s="206">
-        <f>F16/4*2</f>
-        <v>0</v>
-      </c>
-      <c r="G17" s="197" t="s">
-        <v>137</v>
-      </c>
-      <c r="J17" s="201" t="s">
-        <v>137</v>
-      </c>
-      <c r="K17" s="201">
-        <f>(K16-K19)/3*2</f>
-        <v>-40</v>
-      </c>
-    </row>
-    <row r="18" spans="2:15">
-      <c r="B18" s="197"/>
-      <c r="C18" s="198"/>
-      <c r="D18" s="197"/>
-      <c r="E18" s="197"/>
-      <c r="F18" s="206">
-        <f>F16/4</f>
-        <v>0</v>
-      </c>
-      <c r="G18" s="197" t="s">
-        <v>138</v>
-      </c>
-      <c r="J18" s="201" t="s">
-        <v>138</v>
-      </c>
-      <c r="K18" s="201">
-        <f>(K16-K19)/3</f>
-        <v>-20</v>
-      </c>
+      <c r="K18" s="23">
+        <f>F18</f>
+        <v>0</v>
+      </c>
+      <c r="M18" s="23"/>
+      <c r="N18" s="23"/>
+      <c r="O18" s="23"/>
     </row>
     <row r="19" spans="2:15">
       <c r="B19" s="197"/>
       <c r="C19" s="198"/>
       <c r="D19" s="197"/>
-      <c r="E19" s="192">
-        <f>F19</f>
-        <v>0</v>
-      </c>
-      <c r="F19" s="193">
-        <f>F16/4</f>
+      <c r="E19" s="197"/>
+      <c r="F19" s="206">
+        <f>F18/4*2</f>
         <v>0</v>
       </c>
       <c r="G19" s="197" t="s">
-        <v>282</v>
+        <v>136</v>
       </c>
       <c r="J19" s="201" t="s">
-        <v>282</v>
-      </c>
-      <c r="K19" s="211">
-        <v>60</v>
+        <v>136</v>
+      </c>
+      <c r="K19" s="201">
+        <f>(K18-K21)/3*2</f>
+        <v>-40</v>
       </c>
     </row>
     <row r="20" spans="2:15">
       <c r="B20" s="197"/>
       <c r="C20" s="198"/>
       <c r="D20" s="197"/>
-      <c r="E20" s="206">
-        <f>E19/5*2</f>
-        <v>0</v>
-      </c>
-      <c r="F20" s="197" t="s">
+      <c r="E20" s="197"/>
+      <c r="F20" s="206">
+        <f>F18/4</f>
+        <v>0</v>
+      </c>
+      <c r="G20" s="197" t="s">
         <v>137</v>
       </c>
-      <c r="G20" s="197"/>
+      <c r="J20" s="201" t="s">
+        <v>137</v>
+      </c>
+      <c r="K20" s="201">
+        <f>(K18-K21)/3</f>
+        <v>-20</v>
+      </c>
     </row>
     <row r="21" spans="2:15">
       <c r="B21" s="197"/>
       <c r="C21" s="198"/>
       <c r="D21" s="197"/>
-      <c r="E21" s="206">
-        <f>E19/5*2</f>
-        <v>0</v>
-      </c>
-      <c r="F21" s="197" t="s">
-        <v>138</v>
-      </c>
-      <c r="G21" s="197"/>
+      <c r="E21" s="192">
+        <f>F21</f>
+        <v>0</v>
+      </c>
+      <c r="F21" s="193">
+        <f>F18/4</f>
+        <v>0</v>
+      </c>
+      <c r="G21" s="197" t="s">
+        <v>279</v>
+      </c>
+      <c r="J21" s="201" t="s">
+        <v>279</v>
+      </c>
+      <c r="K21" s="211">
+        <v>60</v>
+      </c>
     </row>
     <row r="22" spans="2:15">
       <c r="B22" s="197"/>
       <c r="C22" s="198"/>
-      <c r="D22" s="192">
-        <f>E22</f>
-        <v>0</v>
-      </c>
-      <c r="E22" s="193">
-        <f>E19/5</f>
+      <c r="D22" s="197"/>
+      <c r="E22" s="206">
+        <f>E21/5*2</f>
         <v>0</v>
       </c>
       <c r="F22" s="197" t="s">
-        <v>282</v>
+        <v>136</v>
       </c>
       <c r="G22" s="197"/>
     </row>
     <row r="23" spans="2:15">
       <c r="B23" s="197"/>
       <c r="C23" s="198"/>
-      <c r="D23" s="206">
-        <f>D22/5*2</f>
-        <v>0</v>
-      </c>
-      <c r="E23" s="197" t="s">
+      <c r="D23" s="197"/>
+      <c r="E23" s="206">
+        <f>E21/5*2</f>
+        <v>0</v>
+      </c>
+      <c r="F23" s="197" t="s">
         <v>137</v>
       </c>
-      <c r="F23" s="197"/>
       <c r="G23" s="197"/>
     </row>
     <row r="24" spans="2:15">
       <c r="B24" s="197"/>
       <c r="C24" s="198"/>
-      <c r="D24" s="206">
-        <f>D22/5*2</f>
-        <v>0</v>
-      </c>
-      <c r="E24" s="197" t="s">
-        <v>138</v>
-      </c>
-      <c r="F24" s="197"/>
+      <c r="D24" s="192">
+        <f>E24</f>
+        <v>0</v>
+      </c>
+      <c r="E24" s="193">
+        <f>E21/5</f>
+        <v>0</v>
+      </c>
+      <c r="F24" s="197" t="s">
+        <v>279</v>
+      </c>
       <c r="G24" s="197"/>
     </row>
     <row r="25" spans="2:15">
       <c r="B25" s="197"/>
       <c r="C25" s="198"/>
       <c r="D25" s="206">
-        <f>D22/5</f>
+        <f>D24/5*2</f>
         <v>0</v>
       </c>
       <c r="E25" s="197" t="s">
-        <v>282</v>
+        <v>136</v>
       </c>
       <c r="F25" s="197"/>
       <c r="G25" s="197"/>
     </row>
     <row r="26" spans="2:15">
-      <c r="C26" s="156"/>
+      <c r="B26" s="197"/>
+      <c r="C26" s="198"/>
+      <c r="D26" s="206">
+        <f>D24/5*2</f>
+        <v>0</v>
+      </c>
+      <c r="E26" s="197" t="s">
+        <v>137</v>
+      </c>
+      <c r="F26" s="197"/>
+      <c r="G26" s="197"/>
     </row>
     <row r="27" spans="2:15">
-      <c r="C27" s="156"/>
+      <c r="B27" s="197"/>
+      <c r="C27" s="198"/>
+      <c r="D27" s="206">
+        <f>D24/5</f>
+        <v>0</v>
+      </c>
+      <c r="E27" s="197" t="s">
+        <v>279</v>
+      </c>
+      <c r="F27" s="197"/>
+      <c r="G27" s="197"/>
     </row>
     <row r="28" spans="2:15">
       <c r="C28" s="156"/>
-      <c r="D28" s="203" t="s">
-        <v>291</v>
-      </c>
-      <c r="E28" s="204" t="s">
+    </row>
+    <row r="29" spans="2:15">
+      <c r="C29" s="156"/>
+    </row>
+    <row r="30" spans="2:15">
+      <c r="C30" s="156"/>
+      <c r="D30" s="203" t="s">
+        <v>288</v>
+      </c>
+      <c r="E30" s="204" t="s">
+        <v>286</v>
+      </c>
+      <c r="F30" s="204" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="31" spans="2:15">
+      <c r="B31" s="185" t="s">
+        <v>282</v>
+      </c>
+      <c r="C31" s="200" t="s">
+        <v>277</v>
+      </c>
+      <c r="D31" s="185"/>
+      <c r="E31" s="207"/>
+      <c r="F31" s="186">
+        <f>G31</f>
+        <v>0</v>
+      </c>
+      <c r="G31" s="186">
+        <f>$D$13</f>
+        <v>0</v>
+      </c>
+      <c r="H31" s="23" t="s">
+        <v>278</v>
+      </c>
+      <c r="I31" s="23"/>
+      <c r="J31" s="23" t="s">
         <v>289</v>
       </c>
-      <c r="F28" s="204" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="29" spans="2:15">
-      <c r="B29" s="185" t="s">
-        <v>285</v>
-      </c>
-      <c r="C29" s="200" t="s">
-        <v>280</v>
-      </c>
-      <c r="D29" s="185"/>
-      <c r="E29" s="207"/>
-      <c r="F29" s="186">
-        <f>G29</f>
-        <v>0</v>
-      </c>
-      <c r="G29" s="186">
-        <f>$D$11</f>
-        <v>0</v>
-      </c>
-      <c r="H29" s="23" t="s">
-        <v>281</v>
-      </c>
-      <c r="I29" s="23"/>
-      <c r="J29" s="23" t="s">
-        <v>292</v>
-      </c>
-      <c r="K29" s="23">
-        <f>F29</f>
-        <v>0</v>
-      </c>
-      <c r="L29" s="23"/>
-      <c r="M29" s="23"/>
-      <c r="N29" s="23"/>
-      <c r="O29" s="23"/>
-    </row>
-    <row r="30" spans="2:15">
-      <c r="B30" s="187"/>
-      <c r="C30" s="196"/>
-      <c r="D30" s="187"/>
-      <c r="E30" s="197"/>
-      <c r="F30" s="206">
-        <f>F29/5*2</f>
-        <v>0</v>
-      </c>
-      <c r="G30" s="197" t="s">
-        <v>137</v>
-      </c>
-      <c r="J30" s="201" t="s">
-        <v>137</v>
-      </c>
-      <c r="K30" s="201">
-        <f>(K29-K32)/4*2</f>
+      <c r="K31" s="23">
+        <f>F31</f>
+        <v>0</v>
+      </c>
+      <c r="L31" s="23"/>
+      <c r="M31" s="23"/>
+      <c r="N31" s="23"/>
+      <c r="O31" s="23"/>
+    </row>
+    <row r="32" spans="2:15">
+      <c r="B32" s="187"/>
+      <c r="C32" s="196"/>
+      <c r="D32" s="187"/>
+      <c r="E32" s="197"/>
+      <c r="F32" s="206">
+        <f>F31/5*2</f>
+        <v>0</v>
+      </c>
+      <c r="G32" s="197" t="s">
+        <v>136</v>
+      </c>
+      <c r="J32" s="201" t="s">
+        <v>136</v>
+      </c>
+      <c r="K32" s="201">
+        <f>(K31-K34)/4*2</f>
         <v>-40</v>
       </c>
     </row>
-    <row r="31" spans="2:15">
-      <c r="B31" s="197"/>
-      <c r="C31" s="198"/>
-      <c r="D31" s="197"/>
-      <c r="E31" s="197"/>
-      <c r="F31" s="206">
-        <f>F29/5*2</f>
-        <v>0</v>
-      </c>
-      <c r="G31" s="197" t="s">
-        <v>138</v>
-      </c>
-      <c r="J31" s="201" t="s">
-        <v>138</v>
-      </c>
-      <c r="K31" s="201">
-        <f>(K29-K32)/4*2</f>
-        <v>-40</v>
-      </c>
-    </row>
-    <row r="32" spans="2:15">
-      <c r="B32" s="197"/>
-      <c r="C32" s="198"/>
-      <c r="D32" s="197"/>
-      <c r="E32" s="188">
-        <f>F32</f>
-        <v>0</v>
-      </c>
-      <c r="F32" s="189">
-        <f>F29/5</f>
-        <v>0</v>
-      </c>
-      <c r="G32" s="197" t="s">
-        <v>282</v>
-      </c>
-      <c r="J32" s="201" t="s">
-        <v>282</v>
-      </c>
-      <c r="K32" s="211">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="33" spans="2:7">
+    <row r="33" spans="2:11">
       <c r="B33" s="197"/>
       <c r="C33" s="198"/>
       <c r="D33" s="197"/>
-      <c r="E33" s="206">
-        <f>E32/5*2</f>
-        <v>0</v>
-      </c>
-      <c r="F33" s="197" t="s">
+      <c r="E33" s="197"/>
+      <c r="F33" s="206">
+        <f>F31/5*2</f>
+        <v>0</v>
+      </c>
+      <c r="G33" s="197" t="s">
         <v>137</v>
       </c>
-      <c r="G33" s="197"/>
-    </row>
-    <row r="34" spans="2:7">
+      <c r="J33" s="201" t="s">
+        <v>137</v>
+      </c>
+      <c r="K33" s="201">
+        <f>(K31-K34)/4*2</f>
+        <v>-40</v>
+      </c>
+    </row>
+    <row r="34" spans="2:11">
       <c r="B34" s="197"/>
       <c r="C34" s="198"/>
       <c r="D34" s="197"/>
-      <c r="E34" s="206">
-        <f>E32/5*2</f>
-        <v>0</v>
-      </c>
-      <c r="F34" s="197" t="s">
-        <v>138</v>
-      </c>
-      <c r="G34" s="197"/>
-    </row>
-    <row r="35" spans="2:7">
-      <c r="B35" s="208"/>
-      <c r="C35" s="209"/>
-      <c r="D35" s="188">
-        <f>E35</f>
-        <v>0</v>
-      </c>
-      <c r="E35" s="210">
-        <f>E32/5</f>
-        <v>0</v>
-      </c>
-      <c r="F35" s="208" t="s">
-        <v>282</v>
-      </c>
-      <c r="G35" s="208"/>
-    </row>
-    <row r="36" spans="2:7">
-      <c r="B36" s="198"/>
+      <c r="E34" s="188">
+        <f>F34</f>
+        <v>0</v>
+      </c>
+      <c r="F34" s="189">
+        <f>F31/5</f>
+        <v>0</v>
+      </c>
+      <c r="G34" s="197" t="s">
+        <v>279</v>
+      </c>
+      <c r="J34" s="201" t="s">
+        <v>279</v>
+      </c>
+      <c r="K34" s="211">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="35" spans="2:11">
+      <c r="B35" s="197"/>
+      <c r="C35" s="198"/>
+      <c r="D35" s="197"/>
+      <c r="E35" s="206">
+        <f>E34/5*2</f>
+        <v>0</v>
+      </c>
+      <c r="F35" s="197" t="s">
+        <v>136</v>
+      </c>
+      <c r="G35" s="197"/>
+    </row>
+    <row r="36" spans="2:11">
+      <c r="B36" s="197"/>
       <c r="C36" s="198"/>
-      <c r="D36" s="206">
-        <f>D35/5*2</f>
-        <v>0</v>
-      </c>
-      <c r="E36" s="197" t="s">
+      <c r="D36" s="197"/>
+      <c r="E36" s="206">
+        <f>E34/5*2</f>
+        <v>0</v>
+      </c>
+      <c r="F36" s="197" t="s">
         <v>137</v>
       </c>
-      <c r="F36" s="197"/>
       <c r="G36" s="197"/>
     </row>
-    <row r="37" spans="2:7">
-      <c r="B37" s="198"/>
-      <c r="C37" s="198"/>
-      <c r="D37" s="206">
-        <f>D35/5*2</f>
-        <v>0</v>
-      </c>
-      <c r="E37" s="197" t="s">
-        <v>138</v>
-      </c>
-      <c r="F37" s="197"/>
-      <c r="G37" s="197"/>
-    </row>
-    <row r="38" spans="2:7">
+    <row r="37" spans="2:11">
+      <c r="B37" s="208"/>
+      <c r="C37" s="209"/>
+      <c r="D37" s="188">
+        <f>E37</f>
+        <v>0</v>
+      </c>
+      <c r="E37" s="210">
+        <f>E34/5</f>
+        <v>0</v>
+      </c>
+      <c r="F37" s="208" t="s">
+        <v>279</v>
+      </c>
+      <c r="G37" s="208"/>
+    </row>
+    <row r="38" spans="2:11">
       <c r="B38" s="198"/>
       <c r="C38" s="198"/>
       <c r="D38" s="206">
-        <f>D35/5</f>
-        <v>0</v>
-      </c>
-      <c r="E38" s="208" t="s">
-        <v>282</v>
+        <f>D37/5*2</f>
+        <v>0</v>
+      </c>
+      <c r="E38" s="197" t="s">
+        <v>136</v>
       </c>
       <c r="F38" s="197"/>
       <c r="G38" s="197"/>
+    </row>
+    <row r="39" spans="2:11">
+      <c r="B39" s="198"/>
+      <c r="C39" s="198"/>
+      <c r="D39" s="206">
+        <f>D37/5*2</f>
+        <v>0</v>
+      </c>
+      <c r="E39" s="197" t="s">
+        <v>137</v>
+      </c>
+      <c r="F39" s="197"/>
+      <c r="G39" s="197"/>
+    </row>
+    <row r="40" spans="2:11">
+      <c r="B40" s="198"/>
+      <c r="C40" s="198"/>
+      <c r="D40" s="206">
+        <f>D37/5</f>
+        <v>0</v>
+      </c>
+      <c r="E40" s="208" t="s">
+        <v>279</v>
+      </c>
+      <c r="F40" s="197"/>
+      <c r="G40" s="197"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -10907,19 +10963,19 @@
   <sheetData>
     <row r="1" spans="2:14" s="72" customFormat="1" ht="14">
       <c r="E1" s="73" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F1" s="74" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G1" s="73" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H1" s="74" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I1" s="75" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J1" s="74"/>
       <c r="K1" s="76" t="s">
@@ -10928,23 +10984,23 @@
     </row>
     <row r="2" spans="2:14" s="80" customFormat="1" ht="14">
       <c r="E2" s="81" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F2" s="82" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G2" s="81" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="H2" s="82" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I2" s="83" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="J2" s="82"/>
       <c r="K2" s="84" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="3" spans="2:14">
@@ -10961,10 +11017,10 @@
       <c r="J3" s="45"/>
       <c r="K3" s="43"/>
       <c r="M3" s="23" t="s">
+        <v>112</v>
+      </c>
+      <c r="N3" s="23" t="s">
         <v>113</v>
-      </c>
-      <c r="N3" s="23" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="4" spans="2:14">
@@ -10973,10 +11029,10 @@
         <v>Brioche</v>
       </c>
       <c r="C4" s="62" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D4" s="62" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E4" s="59">
         <f t="shared" ref="E4:E10" si="0">H4</f>
@@ -11016,10 +11072,10 @@
         <v>#REF!</v>
       </c>
       <c r="C5" s="160" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D5" s="160" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E5" s="161" t="e">
         <f t="shared" ref="E5" si="1">H5</f>
@@ -11059,10 +11115,10 @@
         <v>Focaccia Naturale</v>
       </c>
       <c r="C6" s="62" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D6" s="62" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E6" s="59">
         <f t="shared" si="0"/>
@@ -11102,10 +11158,10 @@
         <v>Stockdorf Sourdough</v>
       </c>
       <c r="C7" s="62" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D7" s="62" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E7" s="59">
         <f t="shared" si="0"/>
@@ -11145,10 +11201,10 @@
         <v>Focaccia Pomodorini</v>
       </c>
       <c r="C8" s="62" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D8" s="63" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E8" s="59">
         <f t="shared" si="0"/>
@@ -11188,10 +11244,10 @@
         <v>Spelt Sourdough</v>
       </c>
       <c r="C9" s="62" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D9" s="62" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E9" s="59">
         <f t="shared" si="0"/>
@@ -11231,10 +11287,10 @@
         <v>#REF!</v>
       </c>
       <c r="C10" s="160" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D10" s="160" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E10" s="161" t="e">
         <f t="shared" si="0"/>
@@ -11274,10 +11330,10 @@
         <v>Ciabatta Olive &amp; Origano</v>
       </c>
       <c r="C11" s="62" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D11" s="62" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E11" s="59"/>
       <c r="F11" s="47"/>
@@ -11294,10 +11350,10 @@
         <v>Ciabatta Naturale</v>
       </c>
       <c r="C12" s="62" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D12" s="62" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E12" s="59"/>
       <c r="F12" s="47"/>
@@ -11314,10 +11370,10 @@
         <v>Baguette</v>
       </c>
       <c r="C13" s="62" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D13" s="62" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E13" s="59">
         <f t="shared" ref="E13" si="10">H13</f>
@@ -11357,10 +11413,10 @@
         <v>Pizzaballen (10x 252gr)</v>
       </c>
       <c r="C14" s="62" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D14" s="62" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E14" s="59"/>
       <c r="F14" s="47"/>
@@ -11378,10 +11434,10 @@
         <v>Focaccia Fulvio (2x 30x40)</v>
       </c>
       <c r="C15" s="62" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D15" s="62" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E15" s="59"/>
       <c r="F15" s="47"/>
@@ -11399,10 +11455,10 @@
         <v>Brezen</v>
       </c>
       <c r="C16" s="62" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D16" s="62" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E16" s="59"/>
       <c r="F16" s="47"/>
@@ -11420,10 +11476,10 @@
         <v>Baby brioche</v>
       </c>
       <c r="C17" s="62" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D17" s="62" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E17" s="59">
         <f>H17</f>
@@ -11463,10 +11519,10 @@
         <v>Bagels</v>
       </c>
       <c r="C18" s="62" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D18" s="62" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E18" s="59"/>
       <c r="F18" s="47"/>
@@ -11484,10 +11540,10 @@
         <v>Frühstückssemmel</v>
       </c>
       <c r="C19" s="62" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D19" s="62" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E19" s="59">
         <f t="shared" ref="E19" si="15">H19</f>
@@ -11525,10 +11581,10 @@
         <v>Blechpizza (abends) (1 blech = 2x 252gr)</v>
       </c>
       <c r="C20" s="62" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D20" s="62" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E20" s="59"/>
       <c r="F20" s="47"/>
@@ -11542,13 +11598,13 @@
     </row>
     <row r="23" spans="2:15">
       <c r="B23" s="23" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C23" s="64" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D23" s="64" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E23" s="65">
         <f>H23</f>
@@ -11574,10 +11630,10 @@
     </row>
     <row r="24" spans="2:15">
       <c r="C24" s="64" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D24" s="61" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E24" s="65">
         <f>H24</f>
@@ -11611,16 +11667,16 @@
     </row>
     <row r="28" spans="2:15">
       <c r="H28" s="26" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="I28" s="64" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="J28" s="64" t="s">
+        <v>123</v>
+      </c>
+      <c r="K28" s="64" t="s">
         <v>124</v>
-      </c>
-      <c r="K28" s="64" t="s">
-        <v>125</v>
       </c>
       <c r="L28" s="64" t="s">
         <v>35</v>
@@ -11696,7 +11752,7 @@
         <v>-66.666666666666671</v>
       </c>
       <c r="O30" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="31" spans="2:15">
@@ -11705,7 +11761,7 @@
         <v>-33.333333333333336</v>
       </c>
       <c r="O31" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="32" spans="2:15">
@@ -11713,12 +11769,12 @@
         <v>100</v>
       </c>
       <c r="O32" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="33" spans="2:14">
       <c r="B33" s="71" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="N33" s="55">
         <f>SUM(N30:N32)</f>
@@ -11727,17 +11783,17 @@
     </row>
     <row r="34" spans="2:14">
       <c r="B34" s="71" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="I34" s="55"/>
       <c r="J34" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="35" spans="2:14">
       <c r="I35" s="55"/>
       <c r="J35" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="N35">
         <f>250/3</f>
@@ -11746,7 +11802,7 @@
     </row>
     <row r="36" spans="2:14">
       <c r="J36" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
   </sheetData>
@@ -14134,19 +14190,19 @@
   <sheetData>
     <row r="1" spans="2:17">
       <c r="G1" s="109" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H1" s="118"/>
     </row>
     <row r="2" spans="2:17">
       <c r="B2" s="119" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C2" s="120" t="s">
         <v>60</v>
       </c>
       <c r="D2" s="41" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E2" s="121" t="s">
         <v>1</v>
@@ -14155,10 +14211,10 @@
         <v>58</v>
       </c>
       <c r="G2" s="109" t="s">
+        <v>80</v>
+      </c>
+      <c r="H2" s="123" t="s">
         <v>81</v>
-      </c>
-      <c r="H2" s="123" t="s">
-        <v>82</v>
       </c>
       <c r="K2" s="51" t="s">
         <v>59</v>
@@ -14176,18 +14232,18 @@
         <v>58</v>
       </c>
       <c r="P2" s="49" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="3" spans="2:17">
       <c r="B3" s="132" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C3" t="s">
         <v>54</v>
       </c>
       <c r="D3" s="41" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E3" s="111">
         <v>0.27083333333333331</v>
@@ -14198,10 +14254,10 @@
       <c r="G3" s="112"/>
       <c r="H3" s="124"/>
       <c r="K3" s="130" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="L3" s="133" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="M3" s="134" t="str" cm="1">
         <f t="array" ref="M3">_xlfn.SWITCH(WEEKDAY(($M$2+N3),2),1,"MO",2,"TU",3,"WE",4,"TH",5,"FR",6,"SA",7,"SO")</f>
@@ -14214,18 +14270,18 @@
         <v>0.54166666666666663</v>
       </c>
       <c r="P3" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="4" spans="2:17">
       <c r="B4" s="132" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D4" s="41" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E4" s="111">
         <v>0.29166666666666669</v>
@@ -14236,7 +14292,7 @@
       <c r="G4" s="112"/>
       <c r="H4" s="147"/>
       <c r="K4" s="130" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="L4" s="133" t="s">
         <v>54</v>
@@ -14257,13 +14313,13 @@
     </row>
     <row r="5" spans="2:17">
       <c r="B5" s="132" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C5" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D5" s="41" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E5" s="111">
         <v>0.32291666666666669</v>
@@ -14274,10 +14330,10 @@
       <c r="G5" s="174"/>
       <c r="H5" s="147"/>
       <c r="K5" s="130" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="L5" s="133" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="M5" s="134" t="str" cm="1">
         <f t="array" ref="M5">_xlfn.SWITCH(WEEKDAY(($M$2+N5),2),1,"MO",2,"TU",3,"WE",4,"TH",5,"FR",6,"SA",7,"SO")</f>
@@ -14294,13 +14350,13 @@
     </row>
     <row r="6" spans="2:17">
       <c r="B6" s="132" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D6" s="41" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E6" s="111">
         <v>0.35416666666666669</v>
@@ -14311,7 +14367,7 @@
       <c r="G6" s="112"/>
       <c r="H6" s="123"/>
       <c r="K6" s="130" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="L6" s="133" t="s">
         <v>55</v>
@@ -14331,13 +14387,13 @@
     </row>
     <row r="7" spans="2:17">
       <c r="B7" s="132" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C7" t="s">
         <v>55</v>
       </c>
       <c r="D7" s="41" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E7" s="111">
         <v>0.41666666666666669</v>
@@ -14347,10 +14403,10 @@
       </c>
       <c r="G7" s="112"/>
       <c r="K7" s="130" t="s">
+        <v>170</v>
+      </c>
+      <c r="L7" s="133" t="s">
         <v>171</v>
-      </c>
-      <c r="L7" s="133" t="s">
-        <v>172</v>
       </c>
       <c r="M7" s="134" t="str" cm="1">
         <f t="array" ref="M7">_xlfn.SWITCH(WEEKDAY(($M$2+N7),2),1,"MO",2,"TU",3,"WE",4,"TH",5,"FR",6,"SA",7,"SO")</f>
@@ -14367,13 +14423,13 @@
     </row>
     <row r="8" spans="2:17">
       <c r="B8" s="132" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C8" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D8" s="41" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E8" s="111">
         <v>0.4375</v>
@@ -14384,10 +14440,10 @@
       <c r="G8" s="112"/>
       <c r="H8" s="147"/>
       <c r="K8" s="130" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="L8" s="133" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="M8" s="134" t="str" cm="1">
         <f t="array" ref="M8">_xlfn.SWITCH(WEEKDAY(($M$2+N8),2),1,"MO",2,"TU",3,"WE",4,"TH",5,"FR",6,"SA",7,"SO")</f>
@@ -14404,13 +14460,13 @@
     </row>
     <row r="9" spans="2:17">
       <c r="B9" s="132" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C9" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D9" s="41" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E9" s="111">
         <v>0.4548611111111111</v>
@@ -14422,7 +14478,7 @@
       <c r="H9" s="147"/>
       <c r="I9" s="78"/>
       <c r="K9" s="130" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="L9" s="133" t="s">
         <v>56</v>
@@ -14440,13 +14496,13 @@
     </row>
     <row r="10" spans="2:17">
       <c r="B10" s="148" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C10" s="79" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D10" s="41" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E10" s="50">
         <v>0.52083333333333337</v>
@@ -14456,10 +14512,10 @@
       </c>
       <c r="G10" s="112"/>
       <c r="K10" s="132" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="L10" s="133" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="M10" s="134" t="str" cm="1">
         <f t="array" ref="M10">_xlfn.SWITCH(WEEKDAY(($M$2+N10),2),1,"MO",2,"TU",3,"WE",4,"TH",5,"FR",6,"SA",7,"SO")</f>
@@ -14476,13 +14532,13 @@
     </row>
     <row r="11" spans="2:17">
       <c r="B11" s="131" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C11" s="79" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D11" s="41" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E11" s="53">
         <v>0.52083333333333337</v>
@@ -14493,7 +14549,7 @@
       <c r="G11" s="112"/>
       <c r="H11" s="147"/>
       <c r="K11" s="132" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="L11" s="133" t="s">
         <v>54</v>
@@ -14512,13 +14568,13 @@
     </row>
     <row r="12" spans="2:17">
       <c r="B12" s="148" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C12" s="79" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="D12" s="41" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E12" s="50">
         <v>0.54166666666666663</v>
@@ -14529,10 +14585,10 @@
       <c r="G12" s="112"/>
       <c r="I12" s="78"/>
       <c r="K12" s="132" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="L12" s="133" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="M12" s="134" t="str" cm="1">
         <f t="array" ref="M12">_xlfn.SWITCH(WEEKDAY(($M$2+N12),2),1,"MO",2,"TU",3,"WE",4,"TH",5,"FR",6,"SA",7,"SO")</f>
@@ -14549,13 +14605,13 @@
     </row>
     <row r="13" spans="2:17">
       <c r="B13" s="131" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C13" s="79" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="D13" s="41" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E13" s="50">
         <v>0.54166666666666663</v>
@@ -14566,10 +14622,10 @@
       <c r="G13" s="112"/>
       <c r="H13" s="147"/>
       <c r="K13" s="132" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="L13" s="133" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="M13" s="134" t="str" cm="1">
         <f t="array" ref="M13">_xlfn.SWITCH(WEEKDAY(($M$2+N13),2),1,"MO",2,"TU",3,"WE",4,"TH",5,"FR",6,"SA",7,"SO")</f>
@@ -14586,13 +14642,13 @@
     </row>
     <row r="14" spans="2:17">
       <c r="B14" s="131" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C14" s="79" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="D14" s="41" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E14" s="53">
         <v>0.54513888888888884</v>
@@ -14604,10 +14660,10 @@
       <c r="H14" s="147"/>
       <c r="J14" s="125"/>
       <c r="K14" s="132" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="L14" s="133" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="M14" s="134" t="str" cm="1">
         <f t="array" ref="M14">_xlfn.SWITCH(WEEKDAY(($M$2+N14),2),1,"MO",2,"TU",3,"WE",4,"TH",5,"FR",6,"SA",7,"SO")</f>
@@ -14624,13 +14680,13 @@
     </row>
     <row r="15" spans="2:17">
       <c r="B15" s="148" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C15" s="79" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D15" s="41" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E15" s="50">
         <v>0.57638888888888884</v>
@@ -14642,7 +14698,7 @@
       <c r="H15" s="147"/>
       <c r="I15" s="78"/>
       <c r="K15" s="132" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="L15" s="133" t="s">
         <v>55</v>
@@ -14663,13 +14719,13 @@
     </row>
     <row r="16" spans="2:17">
       <c r="B16" s="148" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C16" s="79" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D16" s="41" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E16" s="50">
         <v>0.58333333333333337</v>
@@ -14681,10 +14737,10 @@
       <c r="H16" s="147"/>
       <c r="I16" s="78"/>
       <c r="K16" s="132" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="L16" s="133" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="M16" s="134" t="str" cm="1">
         <f t="array" ref="M16">_xlfn.SWITCH(WEEKDAY(($M$2+N16),2),1,"MO",2,"TU",3,"WE",4,"TH",5,"FR",6,"SA",7,"SO")</f>
@@ -14702,13 +14758,13 @@
     </row>
     <row r="17" spans="2:16">
       <c r="B17" s="148" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C17" s="79" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="D17" s="41" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E17" s="50">
         <v>0.60416666666666663</v>
@@ -14718,10 +14774,10 @@
       </c>
       <c r="G17" s="112"/>
       <c r="K17" s="132" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="L17" s="133" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="M17" s="134" t="str" cm="1">
         <f t="array" ref="M17">_xlfn.SWITCH(WEEKDAY(($M$2+N17),2),1,"MO",2,"TU",3,"WE",4,"TH",5,"FR",6,"SA",7,"SO")</f>
@@ -14735,18 +14791,18 @@
         <v>0.625</v>
       </c>
       <c r="P17" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="18" spans="2:16">
       <c r="B18" s="131" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C18" s="79" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D18" s="41" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E18" s="53">
         <v>0.60486111111111107</v>
@@ -14756,10 +14812,10 @@
       </c>
       <c r="G18" s="112"/>
       <c r="K18" s="132" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="L18" s="133" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="M18" s="134" t="str" cm="1">
         <f t="array" ref="M18">_xlfn.SWITCH(WEEKDAY(($M$2+N18),2),1,"MO",2,"TU",3,"WE",4,"TH",5,"FR",6,"SA",7,"SO")</f>
@@ -14776,13 +14832,13 @@
     </row>
     <row r="19" spans="2:16">
       <c r="B19" s="148" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C19" s="79" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="D19" s="41" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E19" s="50">
         <v>0.61805555555555558</v>
@@ -14793,7 +14849,7 @@
       <c r="G19" s="112"/>
       <c r="H19" s="147"/>
       <c r="K19" s="132" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="L19" s="133" t="s">
         <v>56</v>
@@ -14811,13 +14867,13 @@
     </row>
     <row r="20" spans="2:16">
       <c r="B20" s="131" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C20" s="79" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D20" s="41" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E20" s="53">
         <v>0.625</v>
@@ -14828,7 +14884,7 @@
       <c r="G20" s="112"/>
       <c r="H20" s="147"/>
       <c r="K20" s="142" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="L20" s="138" t="s">
         <v>57</v>
@@ -14847,13 +14903,13 @@
     </row>
     <row r="21" spans="2:16">
       <c r="B21" s="148" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C21" s="79" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D21" s="41" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E21" s="50">
         <v>0.63194444444444442</v>
@@ -14865,10 +14921,10 @@
       <c r="H21" s="147"/>
       <c r="J21" s="125"/>
       <c r="K21" s="142" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="L21" s="138" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="M21" s="134" t="str" cm="1">
         <f t="array" ref="M21">_xlfn.SWITCH(WEEKDAY(($M$2+N21),2),1,"MO",2,"TU",3,"WE",4,"TH",5,"FR",6,"SA",7,"SO")</f>
@@ -14885,13 +14941,13 @@
     </row>
     <row r="22" spans="2:16">
       <c r="B22" s="131" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C22" s="79" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="D22" s="41" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E22" s="111">
         <v>0.63888888888888884</v>
@@ -14903,10 +14959,10 @@
       <c r="H22" s="147"/>
       <c r="J22" s="125"/>
       <c r="K22" s="142" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="L22" s="138" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="M22" s="134" t="str" cm="1">
         <f t="array" ref="M22">_xlfn.SWITCH(WEEKDAY(($M$2+N22),2),1,"MO",2,"TU",3,"WE",4,"TH",5,"FR",6,"SA",7,"SO")</f>
@@ -14920,18 +14976,18 @@
         <v>0.51736111111111116</v>
       </c>
       <c r="P22" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="23" spans="2:16">
       <c r="B23" s="131" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C23" s="79" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D23" s="41" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E23" s="111">
         <v>0.65277777777777779</v>
@@ -14941,10 +14997,10 @@
       </c>
       <c r="G23" s="112"/>
       <c r="K23" s="142" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="L23" s="138" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="M23" s="134" t="str" cm="1">
         <f t="array" ref="M23">_xlfn.SWITCH(WEEKDAY(($M$2+N23),2),1,"MO",2,"TU",3,"WE",4,"TH",5,"FR",6,"SA",7,"SO")</f>
@@ -14961,13 +15017,13 @@
     </row>
     <row r="24" spans="2:16">
       <c r="B24" s="143" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C24" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="D24" s="41" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E24" s="111">
         <v>0.6875</v>
@@ -14976,10 +15032,10 @@
         <v>1.0416666666666666E-2</v>
       </c>
       <c r="K24" s="142" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="L24" s="138" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="M24" s="134" t="str" cm="1">
         <f t="array" ref="M24">_xlfn.SWITCH(WEEKDAY(($M$2+N24),2),1,"MO",2,"TU",3,"WE",4,"TH",5,"FR",6,"SA",7,"SO")</f>
@@ -14996,13 +15052,13 @@
     </row>
     <row r="25" spans="2:16">
       <c r="B25" s="143" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C25" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="D25" s="41" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E25" s="111">
         <v>0.69791666666666663</v>
@@ -15013,10 +15069,10 @@
       <c r="G25" s="112"/>
       <c r="H25" s="147"/>
       <c r="K25" s="142" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="L25" s="138" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="M25" s="134" t="str" cm="1">
         <f t="array" ref="M25">_xlfn.SWITCH(WEEKDAY(($M$2+N25),2),1,"MO",2,"TU",3,"WE",4,"TH",5,"FR",6,"SA",7,"SO")</f>
@@ -15033,13 +15089,13 @@
     </row>
     <row r="26" spans="2:16">
       <c r="B26" s="143" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C26" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D26" s="41" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E26" s="53">
         <v>0.71875</v>
@@ -15050,7 +15106,7 @@
       <c r="G26" s="112"/>
       <c r="H26" s="147"/>
       <c r="K26" s="142" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="L26" s="138" t="s">
         <v>56</v>
@@ -15068,13 +15124,13 @@
     </row>
     <row r="27" spans="2:16">
       <c r="B27" s="142" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C27" s="79" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="D27" s="41" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E27" s="116">
         <v>0.71944444444444444</v>
@@ -15085,10 +15141,10 @@
       <c r="G27" s="112"/>
       <c r="H27" s="147"/>
       <c r="K27" s="58" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L27" s="133" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="M27" s="134" t="str" cm="1">
         <f t="array" ref="M27">_xlfn.SWITCH(WEEKDAY(($M$2+N27),2),1,"MO",2,"TU",3,"WE",4,"TH",5,"FR",6,"SA",7,"SO")</f>
@@ -15104,13 +15160,13 @@
     </row>
     <row r="28" spans="2:16">
       <c r="B28" s="142" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C28" s="79" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="D28" s="41" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E28" s="111">
         <v>0.75</v>
@@ -15121,10 +15177,10 @@
       <c r="G28" s="112"/>
       <c r="H28" s="147"/>
       <c r="K28" s="58" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L28" s="133" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="M28" s="134" t="str" cm="1">
         <f t="array" ref="M28">_xlfn.SWITCH(WEEKDAY(($M$2+N28),2),1,"MO",2,"TU",3,"WE",4,"TH",5,"FR",6,"SA",7,"SO")</f>
@@ -15138,18 +15194,18 @@
         <v>0.33333333333333331</v>
       </c>
       <c r="P28" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="29" spans="2:16">
       <c r="B29" s="142" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C29" s="79" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D29" s="41" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E29" s="111">
         <v>0.76388888888888884</v>
@@ -15159,10 +15215,10 @@
       </c>
       <c r="G29" s="112"/>
       <c r="K29" s="58" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L29" s="133" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="M29" s="134" t="str" cm="1">
         <f t="array" ref="M29">_xlfn.SWITCH(WEEKDAY(($M$2+N29),2),1,"MO",2,"TU",3,"WE",4,"TH",5,"FR",6,"SA",7,"SO")</f>
@@ -15179,13 +15235,13 @@
     </row>
     <row r="30" spans="2:16">
       <c r="B30" s="143" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C30" s="79" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D30" s="41" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E30" s="53">
         <v>0.80208333333333337</v>
@@ -15195,10 +15251,10 @@
       </c>
       <c r="G30" s="112"/>
       <c r="K30" s="58" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L30" s="133" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="M30" s="134" t="str" cm="1">
         <f t="array" ref="M30">_xlfn.SWITCH(WEEKDAY(($M$2+N30),2),1,"MO",2,"TU",3,"WE",4,"TH",5,"FR",6,"SA",7,"SO")</f>
@@ -15212,18 +15268,18 @@
         <v>0.58333333333333337</v>
       </c>
       <c r="P30" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="31" spans="2:16" ht="17" thickBot="1">
       <c r="B31" s="176" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C31" s="177" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="D31" s="139" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E31" s="140">
         <v>0.91041666666666665</v>
@@ -15232,10 +15288,10 @@
       <c r="G31" s="112"/>
       <c r="H31" s="147"/>
       <c r="K31" s="58" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L31" s="133" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="M31" s="134" t="str" cm="1">
         <f t="array" ref="M31">_xlfn.SWITCH(WEEKDAY(($M$2+N31),2),1,"MO",2,"TU",3,"WE",4,"TH",5,"FR",6,"SA",7,"SO")</f>
@@ -15252,13 +15308,13 @@
     </row>
     <row r="32" spans="2:16" ht="17" thickTop="1">
       <c r="B32" s="148" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C32" s="57" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D32" s="41" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E32" s="111">
         <v>0.2361111111111111</v>
@@ -15269,10 +15325,10 @@
       <c r="G32" s="112"/>
       <c r="H32" s="53"/>
       <c r="K32" s="108" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="L32" s="138" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="M32" s="134" t="str" cm="1">
         <f t="array" ref="M32">_xlfn.SWITCH(WEEKDAY(($M$2+N32),2),1,"MO",2,"TU",3,"WE",4,"TH",5,"FR",6,"SA",7,"SO")</f>
@@ -15287,13 +15343,13 @@
     </row>
     <row r="33" spans="2:17">
       <c r="B33" s="148" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C33" s="57" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="D33" s="41" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E33" s="111">
         <v>0.25</v>
@@ -15304,10 +15360,10 @@
       <c r="G33" s="169"/>
       <c r="H33" s="124"/>
       <c r="K33" s="108" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="L33" s="138" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="M33" s="134" t="str" cm="1">
         <f t="array" ref="M33">_xlfn.SWITCH(WEEKDAY(($M$2+N33),2),1,"MO",2,"TU",3,"WE",4,"TH",5,"FR",6,"SA",7,"SO")</f>
@@ -15323,13 +15379,13 @@
     </row>
     <row r="34" spans="2:17">
       <c r="B34" s="131" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C34" s="79" t="s">
         <v>55</v>
       </c>
       <c r="D34" s="41" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E34" s="111">
         <v>0.2638888888888889</v>
@@ -15340,10 +15396,10 @@
       <c r="G34" s="112"/>
       <c r="H34" s="124"/>
       <c r="K34" s="108" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="L34" s="138" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="M34" s="134" t="str" cm="1">
         <f t="array" ref="M34">_xlfn.SWITCH(WEEKDAY(($M$2+N34),2),1,"MO",2,"TU",3,"WE",4,"TH",5,"FR",6,"SA",7,"SO")</f>
@@ -15359,13 +15415,13 @@
     </row>
     <row r="35" spans="2:17">
       <c r="B35" s="131" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C35" s="79" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="D35" s="41" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E35" s="115">
         <v>0.27430555555555558</v>
@@ -15376,10 +15432,10 @@
       <c r="G35" s="112"/>
       <c r="H35" s="124"/>
       <c r="K35" s="108" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="L35" s="138" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="M35" s="134" t="str" cm="1">
         <f t="array" ref="M35">_xlfn.SWITCH(WEEKDAY(($M$2+N35),2),1,"MO",2,"TU",3,"WE",4,"TH",5,"FR",6,"SA",7,"SO")</f>
@@ -15395,13 +15451,13 @@
     </row>
     <row r="36" spans="2:17">
       <c r="B36" s="143" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C36" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="D36" s="41" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E36" s="50">
         <v>0.33333333333333331</v>
@@ -15411,10 +15467,10 @@
       </c>
       <c r="H36" s="124"/>
       <c r="K36" s="108" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="L36" s="138" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="M36" s="134" t="str" cm="1">
         <f t="array" ref="M36">_xlfn.SWITCH(WEEKDAY(($M$2+N36),2),1,"MO",2,"TU",3,"WE",4,"TH",5,"FR",6,"SA",7,"SO")</f>
@@ -15430,13 +15486,13 @@
     </row>
     <row r="37" spans="2:17">
       <c r="B37" s="148" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C37" s="57" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D37" s="41" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E37" s="111">
         <v>0.27500000000000002</v>
@@ -15446,10 +15502,10 @@
       </c>
       <c r="G37" s="169"/>
       <c r="K37" s="108" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="L37" s="138" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="M37" s="134" t="str" cm="1">
         <f t="array" ref="M37">_xlfn.SWITCH(WEEKDAY(($M$2+N37),2),1,"MO",2,"TU",3,"WE",4,"TH",5,"FR",6,"SA",7,"SO")</f>
@@ -15463,18 +15519,18 @@
         <v>0.59375</v>
       </c>
       <c r="P37" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="38" spans="2:17">
       <c r="B38" s="148" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C38" s="57" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="D38" s="41" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E38" s="111">
         <v>0.28472222222222221</v>
@@ -15485,7 +15541,7 @@
       <c r="G38" s="112"/>
       <c r="H38" s="124"/>
       <c r="K38" s="108" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="L38" t="s">
         <v>55</v>
@@ -15504,13 +15560,13 @@
     </row>
     <row r="39" spans="2:17">
       <c r="B39" s="131" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C39" s="155" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D39" s="41" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E39" s="111">
         <v>0.29166666666666669</v>
@@ -15519,10 +15575,10 @@
         <v>2.0833333333333332E-2</v>
       </c>
       <c r="K39" s="108" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="L39" s="138" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="M39" s="134" t="str" cm="1">
         <f t="array" ref="M39">_xlfn.SWITCH(WEEKDAY(($M$2+N39),2),1,"MO",2,"TU",3,"WE",4,"TH",5,"FR",6,"SA",7,"SO")</f>
@@ -15538,13 +15594,13 @@
     </row>
     <row r="40" spans="2:17">
       <c r="B40" s="131" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C40" s="79" t="s">
         <v>56</v>
       </c>
       <c r="D40" s="41" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E40" s="111">
         <v>0.3125</v>
@@ -15553,10 +15609,10 @@
       <c r="G40" s="174"/>
       <c r="H40" s="124"/>
       <c r="K40" s="108" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="L40" s="138" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="M40" s="134" t="str" cm="1">
         <f t="array" ref="M40">_xlfn.SWITCH(WEEKDAY(($M$2+N40),2),1,"MO",2,"TU",3,"WE",4,"TH",5,"FR",6,"SA",7,"SO")</f>
@@ -15572,13 +15628,13 @@
     </row>
     <row r="41" spans="2:17">
       <c r="B41" s="142" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C41" s="79" t="s">
         <v>55</v>
       </c>
       <c r="D41" s="41" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E41" s="111">
         <v>0.31597222222222221</v>
@@ -15587,7 +15643,7 @@
         <v>3.125E-2</v>
       </c>
       <c r="K41" s="108" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="L41" s="138" t="s">
         <v>56</v>
@@ -15604,13 +15660,13 @@
     </row>
     <row r="42" spans="2:17">
       <c r="B42" s="148" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C42" s="155" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="D42" s="41" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E42" s="111">
         <v>0.3263888888888889</v>
@@ -15620,10 +15676,10 @@
       </c>
       <c r="G42" s="112"/>
       <c r="K42" s="143" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="L42" s="133" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="M42" s="134" t="str" cm="1">
         <f t="array" ref="M42">_xlfn.SWITCH(WEEKDAY(($M$2+N42),2),1,"MO",2,"TU",3,"WE",4,"TH",5,"FR",6,"SA",7,"SO")</f>
@@ -15638,13 +15694,13 @@
     </row>
     <row r="43" spans="2:17">
       <c r="B43" s="142" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C43" s="79" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="D43" s="41" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E43" s="111">
         <v>0.34722222222222221</v>
@@ -15654,10 +15710,10 @@
       </c>
       <c r="G43" s="174"/>
       <c r="K43" s="143" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="L43" s="133" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="M43" s="134" t="str" cm="1">
         <f t="array" ref="M43">_xlfn.SWITCH(WEEKDAY(($M$2+N43),2),1,"MO",2,"TU",3,"WE",4,"TH",5,"FR",6,"SA",7,"SO")</f>
@@ -15674,13 +15730,13 @@
     </row>
     <row r="44" spans="2:17">
       <c r="B44" s="132" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C44" s="23" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="D44" s="156" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E44" s="111">
         <v>0.35416666666666669</v>
@@ -15690,10 +15746,10 @@
       </c>
       <c r="H44" s="124"/>
       <c r="K44" s="143" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="L44" s="133" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="M44" s="134" t="str" cm="1">
         <f t="array" ref="M44">_xlfn.SWITCH(WEEKDAY(($M$2+N44),2),1,"MO",2,"TU",3,"WE",4,"TH",5,"FR",6,"SA",7,"SO")</f>
@@ -15709,13 +15765,13 @@
     </row>
     <row r="45" spans="2:17">
       <c r="B45" s="132" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C45" s="79" t="s">
         <v>56</v>
       </c>
       <c r="D45" s="41" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E45" s="50">
         <v>0.35416666666666669</v>
@@ -15723,10 +15779,10 @@
       <c r="F45" s="54"/>
       <c r="G45" s="174"/>
       <c r="K45" s="143" t="s">
+        <v>175</v>
+      </c>
+      <c r="L45" s="133" t="s">
         <v>176</v>
-      </c>
-      <c r="L45" s="133" t="s">
-        <v>177</v>
       </c>
       <c r="M45" s="134" t="str" cm="1">
         <f t="array" ref="M45">_xlfn.SWITCH(WEEKDAY(($M$2+N45),2),1,"MO",2,"TU",3,"WE",4,"TH",5,"FR",6,"SA",7,"SO")</f>
@@ -15742,13 +15798,13 @@
     </row>
     <row r="46" spans="2:17">
       <c r="B46" s="142" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C46" s="79" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D46" s="41" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E46" s="53">
         <v>0.36805555555555558</v>
@@ -15759,10 +15815,10 @@
       <c r="G46" s="112"/>
       <c r="H46" s="124"/>
       <c r="K46" s="143" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="L46" s="133" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="M46" s="134" t="str" cm="1">
         <f t="array" ref="M46">_xlfn.SWITCH(WEEKDAY(($M$2+N46),2),1,"MO",2,"TU",3,"WE",4,"TH",5,"FR",6,"SA",7,"SO")</f>
@@ -15778,13 +15834,13 @@
     </row>
     <row r="47" spans="2:17">
       <c r="B47" s="142" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C47" s="149" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D47" s="41" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E47" s="53">
         <v>0.3888888888888889</v>
@@ -15793,7 +15849,7 @@
         <v>2.0833333333333332E-2</v>
       </c>
       <c r="K47" s="143" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="L47" s="133" t="s">
         <v>56</v>
@@ -15810,13 +15866,13 @@
     </row>
     <row r="48" spans="2:17">
       <c r="B48" s="142" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C48" s="79" t="s">
         <v>56</v>
       </c>
       <c r="D48" s="41" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E48" s="53">
         <v>0.40972222222222221</v>
@@ -15824,10 +15880,10 @@
       <c r="F48" s="54"/>
       <c r="H48" s="124"/>
       <c r="K48" s="144" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="L48" s="133" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="M48" s="134" t="str" cm="1">
         <f t="array" ref="M48">_xlfn.SWITCH(WEEKDAY(($M$2+N48),2),1,"MO",2,"TU",3,"WE",4,"TH",5,"FR",6,"SA",7,"SO")</f>
@@ -15842,13 +15898,13 @@
     </row>
     <row r="49" spans="2:16">
       <c r="B49" s="143" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C49" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="D49" s="41" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E49" s="111">
         <v>0.4375</v>
@@ -15858,10 +15914,10 @@
       </c>
       <c r="H49" s="124"/>
       <c r="K49" s="144" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="L49" s="133" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="M49" s="134" t="str" cm="1">
         <f t="array" ref="M49">_xlfn.SWITCH(WEEKDAY(($M$2+N49),2),1,"MO",2,"TU",3,"WE",4,"TH",5,"FR",6,"SA",7,"SO")</f>
@@ -15877,13 +15933,13 @@
     </row>
     <row r="50" spans="2:16">
       <c r="B50" s="143" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C50" s="23" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="D50" s="41" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E50" s="116">
         <v>0.45833333333333331</v>
@@ -15892,10 +15948,10 @@
         <v>3.125E-2</v>
       </c>
       <c r="K50" s="144" t="s">
+        <v>177</v>
+      </c>
+      <c r="L50" s="133" t="s">
         <v>178</v>
-      </c>
-      <c r="L50" s="133" t="s">
-        <v>179</v>
       </c>
       <c r="M50" s="134" t="str" cm="1">
         <f t="array" ref="M50">_xlfn.SWITCH(WEEKDAY(($M$2+N50),2),1,"MO",2,"TU",3,"WE",4,"TH",5,"FR",6,"SA",7,"SO")</f>
@@ -15909,18 +15965,18 @@
         <v>0.4548611111111111</v>
       </c>
       <c r="P50" s="4" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="51" spans="2:16">
       <c r="B51" s="143" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C51" t="s">
         <v>56</v>
       </c>
       <c r="D51" s="41" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E51" s="111">
         <v>0.48958333333333331</v>
@@ -15928,10 +15984,10 @@
       <c r="F51" s="54"/>
       <c r="H51" s="124"/>
       <c r="K51" s="144" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="L51" s="133" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="M51" s="134" t="str" cm="1">
         <f t="array" ref="M51">_xlfn.SWITCH(WEEKDAY(($M$2+N51),2),1,"MO",2,"TU",3,"WE",4,"TH",5,"FR",6,"SA",7,"SO")</f>
@@ -15953,10 +16009,10 @@
       <c r="F52" s="54"/>
       <c r="H52" s="124"/>
       <c r="K52" s="144" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="L52" s="133" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="M52" s="134" t="str" cm="1">
         <f t="array" ref="M52">_xlfn.SWITCH(WEEKDAY(($M$2+N52),2),1,"MO",2,"TU",3,"WE",4,"TH",5,"FR",6,"SA",7,"SO")</f>
@@ -15979,10 +16035,10 @@
       <c r="G53" s="112"/>
       <c r="H53" s="124"/>
       <c r="K53" s="144" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="L53" s="133" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="M53" s="134" t="str" cm="1">
         <f t="array" ref="M53">_xlfn.SWITCH(WEEKDAY(($M$2+N53),2),1,"MO",2,"TU",3,"WE",4,"TH",5,"FR",6,"SA",7,"SO")</f>
@@ -16004,7 +16060,7 @@
       <c r="F54" s="111"/>
       <c r="H54" s="124"/>
       <c r="K54" s="144" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="L54" s="133" t="s">
         <v>56</v>
@@ -16025,10 +16081,10 @@
       <c r="F55" s="54"/>
       <c r="H55" s="124"/>
       <c r="K55" s="148" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="L55" s="138" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="M55" s="134" t="str" cm="1">
         <f t="array" ref="M55">_xlfn.SWITCH(WEEKDAY(($M$2+N55),2),1,"MO",2,"TU",3,"WE",4,"TH",5,"FR",6,"SA",7,"SO")</f>
@@ -16048,10 +16104,10 @@
       <c r="F56" s="54"/>
       <c r="H56" s="124"/>
       <c r="K56" s="148" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="L56" s="138" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M56" s="134" t="str" cm="1">
         <f t="array" ref="M56">_xlfn.SWITCH(WEEKDAY(($M$2+N56),2),1,"MO",2,"TU",3,"WE",4,"TH",5,"FR",6,"SA",7,"SO")</f>
@@ -16072,10 +16128,10 @@
       <c r="F57" s="54"/>
       <c r="H57" s="124"/>
       <c r="K57" s="148" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="L57" s="138" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="M57" s="134" t="str" cm="1">
         <f t="array" ref="M57">_xlfn.SWITCH(WEEKDAY(($M$2+N57),2),1,"MO",2,"TU",3,"WE",4,"TH",5,"FR",6,"SA",7,"SO")</f>
@@ -16097,10 +16153,10 @@
       <c r="F58" s="54"/>
       <c r="H58" s="124"/>
       <c r="K58" s="148" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="L58" s="138" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="M58" s="134" t="str" cm="1">
         <f t="array" ref="M58">_xlfn.SWITCH(WEEKDAY(($M$2+N58),2),1,"MO",2,"TU",3,"WE",4,"TH",5,"FR",6,"SA",7,"SO")</f>
@@ -16123,10 +16179,10 @@
       <c r="G59" s="112"/>
       <c r="H59" s="124"/>
       <c r="K59" s="148" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="L59" s="138" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="M59" s="134" t="str" cm="1">
         <f t="array" ref="M59">_xlfn.SWITCH(WEEKDAY(($M$2+N59),2),1,"MO",2,"TU",3,"WE",4,"TH",5,"FR",6,"SA",7,"SO")</f>
@@ -16140,7 +16196,7 @@
         <v>0.55208333333333337</v>
       </c>
       <c r="P59" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="60" spans="2:16">
@@ -16150,10 +16206,10 @@
       <c r="F60" s="54"/>
       <c r="G60" s="112"/>
       <c r="K60" s="148" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="L60" s="138" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="M60" s="134" t="str" cm="1">
         <f t="array" ref="M60">_xlfn.SWITCH(WEEKDAY(($M$2+N60),2),1,"MO",2,"TU",3,"WE",4,"TH",5,"FR",6,"SA",7,"SO")</f>
@@ -16176,10 +16232,10 @@
       <c r="G61" s="112"/>
       <c r="H61" s="147"/>
       <c r="K61" s="148" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="L61" s="138" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="M61" s="134" t="str" cm="1">
         <f t="array" ref="M61">_xlfn.SWITCH(WEEKDAY(($M$2+N61),2),1,"MO",2,"TU",3,"WE",4,"TH",5,"FR",6,"SA",7,"SO")</f>
@@ -16193,7 +16249,7 @@
         <v>2.0833333333333332E-2</v>
       </c>
       <c r="P61" s="3" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="62" spans="2:16">
@@ -16204,10 +16260,10 @@
       <c r="F62" s="54"/>
       <c r="G62" s="112"/>
       <c r="K62" s="148" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="L62" s="138" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="M62" s="134" t="str" cm="1">
         <f t="array" ref="M62">_xlfn.SWITCH(WEEKDAY(($M$2+N62),2),1,"MO",2,"TU",3,"WE",4,"TH",5,"FR",6,"SA",7,"SO")</f>
@@ -16228,13 +16284,13 @@
       <c r="E63" s="50"/>
       <c r="F63" s="54"/>
       <c r="G63" s="150" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="K63" s="148" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="L63" s="138" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="M63" s="134" t="str" cm="1">
         <f t="array" ref="M63">_xlfn.SWITCH(WEEKDAY(($M$2+N63),2),1,"MO",2,"TU",3,"WE",4,"TH",5,"FR",6,"SA",7,"SO")</f>
@@ -16259,10 +16315,10 @@
       <c r="F64" s="54"/>
       <c r="G64"/>
       <c r="K64" s="148" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="L64" s="138" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="M64" s="134" t="str" cm="1">
         <f t="array" ref="M64">_xlfn.SWITCH(WEEKDAY(($M$2+N64),2),1,"MO",2,"TU",3,"WE",4,"TH",5,"FR",6,"SA",7,"SO")</f>
@@ -16284,10 +16340,10 @@
       <c r="E65" s="50"/>
       <c r="F65" s="54"/>
       <c r="G65" s="157" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="K65" s="148" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="L65" s="133" t="s">
         <v>56</v>
@@ -16309,7 +16365,7 @@
       <c r="E66" s="111"/>
       <c r="F66" s="54"/>
       <c r="G66" s="158" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="67" spans="2:16" ht="18">
@@ -16318,148 +16374,148 @@
       <c r="E67" s="50"/>
       <c r="F67" s="54"/>
       <c r="G67" s="158" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="68" spans="2:16" ht="18">
       <c r="G68" s="158" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="69" spans="2:16" ht="18">
       <c r="G69" s="157" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="70" spans="2:16" ht="18">
       <c r="G70" s="158" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="71" spans="2:16" ht="18">
       <c r="G71" s="157" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="72" spans="2:16" ht="18">
       <c r="G72" s="158" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="73" spans="2:16" ht="18">
       <c r="G73" s="157" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="M73" s="78"/>
     </row>
     <row r="74" spans="2:16" ht="18">
       <c r="G74" s="158" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="75" spans="2:16" ht="18">
       <c r="G75" s="157" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="76" spans="2:16" ht="18">
       <c r="G76" s="158" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="77" spans="2:16" ht="18">
       <c r="G77" s="157" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="78" spans="2:16" ht="18">
       <c r="G78" s="158" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="79" spans="2:16" ht="18">
       <c r="G79" s="157" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="80" spans="2:16" ht="18">
       <c r="G80" s="158" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="81" spans="7:7" ht="18">
       <c r="G81" s="157" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="82" spans="7:7" ht="18">
       <c r="G82" s="158" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="83" spans="7:7" ht="18">
       <c r="G83" s="158" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="84" spans="7:7" ht="18">
       <c r="G84" s="157" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="85" spans="7:7" ht="18">
       <c r="G85" s="158" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="86" spans="7:7" ht="18">
       <c r="G86" s="158" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="87" spans="7:7" ht="18">
       <c r="G87" s="158" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="88" spans="7:7" ht="18">
       <c r="G88" s="157" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="89" spans="7:7" ht="18">
       <c r="G89" s="158" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="90" spans="7:7" ht="18">
       <c r="G90" s="157" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="91" spans="7:7" ht="18">
       <c r="G91" s="158" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="92" spans="7:7" ht="18">
       <c r="G92" s="158" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="93" spans="7:7" ht="18">
       <c r="G93" s="157" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="94" spans="7:7" ht="18">
       <c r="G94" s="158" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="95" spans="7:7" ht="18">
       <c r="G95" s="158" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
   </sheetData>

</xml_diff>